<commit_message>
Writing spreadsheets for multiple data samples
</commit_message>
<xml_diff>
--- a/news.xlsx
+++ b/news.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M2"/>
+  <dimension ref="A1:M11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -498,87 +498,1038 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
+          <t>Several people died and dozens were injured after a tram derailed and overturned in Croydon. Five people were left trapped inside the vehicle after it came off the tracks in a tunnel near Sandlilands tram station at around 6am. Three of those trapped have been removed from the tram, which is on its side, but two still remain inside as of 11.30am. British Transport Police confirmed there had been "some loss of life". A spokesman added: "It is too early for us to confirm numbers but we are working hard to assess the ongoing incident and we are continuing to focus on recovery efforts." They later confirmed that the driver of the tram was arrested in connection with the incident. Croydon Tram derailment 8 show all Croydon Tram derailment 1/8 The scene after a tram overturned in Croydon, south London, trapping five people and injuring another 40 Steve Parsons/PA 2/8 Police officers walk the site where the tram overturned Carl Court/Getty Images 3/8 Emergency services were called to the scene just after 6am Twitter/@procrastinateur 4/8 Emergency services close to the location where a tram overturned in Croydon, south London PA 5/8 Emergency services at Sandilands tram station in Croydon Ben Morgan 6/8 A police cordon is in place on Addiscombe Road Ben Morgan 7/8 40 people were injured and five trapped inside the tram Ben Morgan 8/8 Witnesses reported seeing victims stretchered from the tram James Long The London Fire Brigade, which has 70 officers in attendance, said at least 40 people were injured after the tram overturned on a sharp bend. Emergency services were called at 6.10am as torrential rain continued to batter London. Over 50 people were taken to hospital. A Met spokesman said: "Police were called to an overturned tram at 6.10 and officers are in attendance." Scene: this aerial picture shows the tram on its side by the track (BBC/ITN) Hannah Collier, who lives nearby the tram station, said: "Heard a massive crash outside my window, now emergency services everywhere for the overturned tram, hope everyone is ok." The 23-year-old added that she had seen people being carried away on stretchers from the scene of the incident. James Long, who lives metres away from the scene of the incident, told the Standard: "It happened on a sharp bend on the approach to Sandilands tram stop. Carnage: Emergency services inspect the overturned tram (Steve Parsons/PA ) "I've never seen so many emergency services attend a scene." A London Fire Brigade spokesman said they had been called at 6.04am to an overturned tram in a tunnel.    SANDILANDS    Emergency Services are dealing with a serious incident at #Sandilands tram stop. Please avoid the area #Croydoncops pic.twitter.com/xp4RPNxXI5 -- Croydon MPS (@MPSCroydon) November 9, 201 "There are eight fire engines and four fire and rescue crews in attendance," they added. People are being warned to avoid the tram line and the area surrounding Sandilands station in east Croydon, where there is a large police cordon and many emergency vehicles. Heard a massive crash outside my window, now emergency services everywhere for the overturned tram, hope everyone is ok #croydon pic.twitter.com/gxQgnPygEJ -- Hannah Collier (@HannahCollier1) November 9, 2016 Police tell me that people who are worried about loved ones should go to St Mildred's Centre on Bingham Road. Don't have phone number yet -- Gavin Barwell MP (@GavinBarwellMP) November 9, 2016 Miguel John, who was on a bus to Bromley when it stopped by Sandilands tram stop, told the Standard: "The road hadn't been shut off yet but emergency services were already at the scene, this would have been around 6.30am. "By this point more emergency services were flooding to the scene and a police car shut off the road with vehicles being ushered down Elgin Road towards Addiscombe. "But it was obvious it was very, very serious due to the amount of emergency services at the scene. @RachelMirrorVid @DailyMirror here you go, I can't actually see the tram though pic.twitter.com/mwz56sxacI -- Hannah Collier (@HannahCollier1) November 9, 2016 "At first there would have been roughly between six or 10 [vehicles], as time passed a lot more arrived and continued to arrive. "Visibly from where I was about two fire engines, two to three ambulances, several police cars and then more arrived as time went on. "I think that's how everyone knew it was very serious, especially how quickly they acted to shut off the road." Emergency: witnesses reported seeing victims stretchered from the tram (James Long) A London Ambulance Service spokesman said: "We were called at 6.13 to an incident at Addiscombe Road in Croydon. "We have sent a number of resources to the scene including ambulance crews, advanced paramedics and single responders in cars. "We are treating a number of patients." Scene: Police, ambulances and fire engines were in attendance (James Long) Rail safety investigators are reportedly on their way to the scene to begin gathering evidence. A British Transport Police spokesman said: "We are currently on scene at a major incident at Sandilands tram stop in Croydon. "Officers are working to deal with a tram derailment, alongside colleagues from other emergency services. "A number of people are believed to have been injured. People are asked to avoid the area." Rain: there were torrential downpours throughout the night (James Long) Mayor of London Sadiq Khan said: "I am in contact with emergency services and TfL, who are working extremely hard to get the situation under control and treat those who have been injured. My thoughts are with all those involved in this incident. "We are asking people to please visit the TfL website, tfl.gov.uk, for the latest travel information." A Transport for London spokesman said: "We are currently working with the emergency services following a derailment involving a tram in Croydon. "There is currently no service on the tram between Reeves Corner and Addington Village / Harrington Road." Today's is believed to be the first tram crash involving fatalities on board since 1959, when two women passengers and the driver died after a tram caught fire in Glasgow, following a collision with a lorry. London's only tram network operates in the south of the capital, from Wimbledon to Beckenham Junction, Elmers End and New Addington, via Croydon. More than 27 million passengers used the service in 2015/16. The system uses a combination of on-street and segregated running for the 17 miles (27km) of track.</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>tram derailment: Several dead and dozens injured; Five people were left trapped inside</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Croydon; in a tunnel near Sandlilands tram station</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>at around 6am</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Several people; dozens injured</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr"/>
+      <c r="G2" t="inlineStr"/>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>1. A tram derailed and overturned in Croydon, injuring dozens and killing several people.
+2. Five people were trapped inside the vehicle after it came off the tracks in a tunnel near Sandlilands tram station.
+3. Three of the trapped individuals were removed from the tram, but two remained inside as of 11.30am.
+4. The driver of the tram was arrested in connection with the incident.
+5. Emergency services, including police, firefighters, and ambulances, responded to the scene.
+6. Witnesses reported seeing victims being stretchered from the tram.
+7. The London Fire Brigade confirmed that at least 40 people were injured and sent 70 officers to the scene.
+8. Rail safety investigators were reportedly on their way to the scene to gather evidence.
+9. The Metropolitan Police and Transport for London also responded to the incident.
+10. The London Ambulance Service treated a number of patients.
+11. The area surrounding the Sandilands station was cordoned off and people were advised to avoid the tram line.
+12. The</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>United Kingdom, England, Croydon</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>2016-11-09 - The tram overturned and derailed in Croydon, injuring dozens and killing some people.
+2016-11-09 - Police, emergency medical services, and fire brigades were called to the scene.
+2016-11-09 - Rail safety investigators reportedly arrived to begin gathering evidence.
+2016-11-09 - The driver of the tram was arrested in connection with the incident.
+2016-11-09 - London's mayor Sadiq Khan and Transport for London issued statements.</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>1. British Transport Police
+2. Croydon Tram derailment
+3. London Fire Brigade
+4. Met spokesman
+5. London Ambulance Service
+6. Hannah Collier
+7. James Long
+8. London Fire Brigade spokesman
+9. Sandilands tram station
+10. Croydon MPS
+11. Miguel John
+12. Rachel Mirror
+13. Daily Mirror
+14. Sadiq Khan
+15. Transport for London (TfL)</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>1. The tram derailed and overturned, causing it to come off the tracks.
+2. Five people were trapped inside the vehicle.
+3. There was some loss of life.
+4. The driver of the tram was arrested in connection with the incident.
+5. Emergency services were called to the scene to respond to the situation.
+6. The London Fire Brigade, London Ambulance Service, and British Transport Police attended the scene to provide medical treatment and assess the damage.
+7. The incident occurred in a tunnel near Sandlands tram station in Croydon, London.
+8. Rail safety investigators were called to the scene to begin gathering evidence and determine the cause of the accident.
+9. The public was advised to avoid the area and seek alternative transportation.
+10. The emergency response teams worked to remove the trapped people from the tram and provide medical attention to the injured.</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>1. A tram derailed and overturned in Croydon, injuring dozens of people.
+2. Five people were trapped inside the overturned tram.
+3. Emergency services were called to the scene at around 6am.
+4. A police cordon was set up around the area.
+5. Several people died and some were injured in the accident.
+6. The driver of the tram was arrested by the British Transport Police.
+7. London Fire Brigade, London Ambulance Service, and other emergency services responded to the incident.
+8. Witnesses reported seeing injured people being carried away on stretchers from the scene.
+9. The investigation into the cause of the accident is ongoing.
+10. The tram line and the area surrounding Sandilands station in east Croydon were closed to the public.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>The other three people killed have now been named as Donald Collett, Philip Logan and Robert Huxley Click to share on WhatsApp (Opens in new window) Click to share on Facebook (Opens in new window) Click to share on Twitter (Opens in new window) THE three remaining victims of the Croydon tram crash which killed seven people in total have been named by police. They are Donald Collett, 62, from Croydon, and Philip Logan, 52, and 63-year-old Robert Huxley, both from New Addington. British Transport Police 22 Donald Collett, 62, (left) and Philip Logan, 52, (right) died in the accident. A picture of Robert Huxley has not yet been released 22 Left to right: Dorota Rynkiewicz, Mark Smith, Phil Seary and Dane Chinnery Getty Images 22 Rail workers at the site work to fix the track where the tram derailed on Wednesday which saw seven people killed Not known 22 Rail workers at the site work to fix the track where the tram derailed on Wednesday Getty Images 22 A tram carriage covered in tarpaulin is driven away from the scene of the accident on a truck in Croydon The other victims who have already been named on Wednesday were Mark Smith, Dane Chinnery, Phil Seary and Dorota Rynkiewicz. The crashed tram carriages were taken away on the back of two lorries on Saturday morning and repair work on the track has started. British Transport Police said the 100ft-long tram had been split into sections which were craned on to flatbed lorries. All sections have now been taken away from the scene as the Rail Accident Investigation Branch (RAIB) continues its inquiry. Investigators believe the tram was travelling at "significantly higher speeds" than those permitted when it derailed. Getty Images 22 Friends and family of some of the victims marched earlier on Saturday to the site of the crash Getty Images 22 Tributes left for victim Mark Davis near the Sandilands tram stop by the site of the Croydon tram crash Getty Images 22 British Transport Police said Donald Collett, 62, of Croydon; Philip Logan, 52, and Robert Huxley, 63, died in the accident when the tram overturned Six men and one woman died and more than 50 were taken to hospital after the early Wednesday morning crash at a "sharp, left-hand curve" near Sandilands tram stop in South London. A group of up to 100 people on Saturday marched down the road to the spot to pay tribute to the victims of the derailing in south London. A statement from Mr Collett's family read: "Don was a well loved, funny and generous man, who could light up a room with his smile. He is tragically leaving behind a loving family, partner, adored friends and work colleagues. Please rest in peace and know you are truly loved and greatly missed." The family of Mr Logan described him as a "true family man" and a "generous friend". A statement from the family added "Phil was a man with more love compassion and zest for life than words can express. He will be immensely missed by all that knew him." One of the victims of the Croydon tram crash tragedy was due to get married next year. Mark Smith, 35, had planned a summer ceremony with his Lithuanian fiancee Indre Novikovaite, 25, the mother of their 18-month-old son. Enterprise News and Pictures 22 Mark Smith and fiancee Indra Novikovaite with their 18 month old son PA:Press Association 22 Philip was described as a 'gentle giant' PA:Press Association 22 A map of where the crash happened Her brother Osvaldas, 23, told The Sun: "They were planning to get married. My sister is completely devastated by this." Mum-of-two Dorota Rynkiewicz, 35, and grandfather Philip Seary, 57, were yesterday also named as among the seven victims of the disaster. Two cranes were also at the accident site in South London to move the wreckage as it was reported bodies were still trapped inside. Facebook 22 Dorota Rynkiewicz with husband Andrzej Rynkiewicz. Jim Bennett 22 PA:Press Association 22 A one minute's silence was observed by the cenotaph in Croydon to mark the crash The two-carriage tram came off the rails at 50mph on a 12mph bend at around 6am on Wednesday. The driver, 42, has been released on police bail following his arrest on suspicion of manslaughter. Dorota, of New Addington, has two young daughters aged five and seven. She was the only woman to die in the crash. Friends described her as an "amazing mother" who always had a "special smile" on her face. Pal Asma Kazim said: "Dorota was full of life, caring and a funny girl. It is shocking news for us and I still can't believe she has gone." London News Pictures 22 The tram tipped PA:Press Association 22 The family of Philip Seary, 57, have paid tribute to the Crystal Palace fan who died in the crash PA:Press Association 22 Workers at the site of the Croydon tram crash stand during a two minute silence to mark Armistice Day Philip, also of New Addington, was said to be a "gentle giant". He was only on the tram after agreeing to swap shifts with a fellow electrical engineer at the Royal Opera House in Covent Garden. Son-in-law Darren Mimms said: "As Phil was such a kind man he would do anything to help anybody. Related stories 'I WARNED THEM' Passenger claims he warned TfL about possible Croydon tram crash repeatedly 'IT'S RIPPED OUR FAMILY APART' Mum-of-three, football fan and young dad named among victims of Croydon tram crash tram horror What caused Croydon tram derailment and where did it overturn? 'I saw my pal's boot, he was obviously dead' Tram crash survivor tells of horrific scene of death and severed limbs Seized at scene Moment Croydon tram crash driver is arrested on suspicion of manslaughter after doing 50 on 12mph bend ACCIDENT WAITING TO HAPPEN? Croydon tram crash 'almost happened week earlier when one "lifted onto side" at same corner' "It's really hurting his wife. He shouldn't have been on that tram. "If he hadn't have been at work he would have been doing bits and bobs around the house and looking after his granddaughter." Tributes were also paid online to keen fisherman Mark, of Coulsdon. His cousin Tom Smith said on Facebook: "Still cannot believe this is true, the last couple of days have just felt like a nightmare that I'm gonna wake up from. Getty Images 22 Emergency workers continued to work at the scene of the derailed tram PA:Press Association 22 Philip was only on the tram because he had agreed to swap shifts with a colleague SWNS:South West News Service 22 Family and friends of one of the deceased lay flowers near the scene of the tram crash News Group Newspapers Ltd 22 Workers were seen today trying to move the tram which crashed earlier this week PA:Press Association 22 Flowers left at the scene near the tram crash in Croydon "Not only were you my cousin but literally my best friend. The thought that we are all never gonna see you or hear from you again makes me feel sick. "We are all in bits and I just wish you could walk back into your home with that smile on your face and make everyone laugh. "I know I have made new family in Indre Novikovaite and Osvaldas Novikovas but I would give everything if you could come back and join us bro. "See you one day for that catch up we kept talking about." Accident investigators hope to have an interim report ready next week. Cops are said to be probing whether the driver was on his phone or had "blacked out." Cranes to clear wreckage as Croydon tram crash victims named</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>tram crash; Final three Croydon tram crash victims named</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Croydon</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Wednesday</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Donald Collett, 62, from Croydon, and Philip Logan, 52, and 63-year-old Robert Huxley</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>travelling at \u201csignificantly higher speeds\u201d</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr"/>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>1. Three more victims of the Croydon tram crash are named by the police: Donald Collett, Philip Logan, and Robert Huxley.
+2. The three remaining victims are identified as: Donald Collett, Philip Logan, and Robert Huxley.
+3. The identities of the four previously named victims are recapped: Mark Smith, Dane Chinnery, Phil Seary, and Dorota Rynkiewicz.
+4. The crashed tram carriages are removed from the scene by flatbed lorries.
+5. Rail workers begin repairs on the track where the tram derailed.
+6. The investigation continues to determine the cause of the accident, with the belief that the tram was travelling at a significantly higher speed than permitted.
+7. Friends and family of some of the victims march to the site of the crash.
+8. A group of up to 100 people pay tribute to the victims of the derailing in south London.
+9. One of the victims, Mark Smith, was due to get married next year.
+10. Tributes are paid online and offline to the other victims.</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>[England,London,Croydon]</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>2016-11-09 - The Croydon tram crash happened.
+2016-11-12 - The first four victims were named by the police.
+2016-11-13 - The remaining three victims were named by the police.
+2016-11-12 - A group of people marched to the site of the crash to pay tribute to the victims.
+2016-11-13 - The bodies of the deceased were taken away by lorries.
+2016-11-11 - One of the victims, Mark Smith, was due to get married next year.
+2016-11-14 - A one-minute silence was observed by the cenotaph in Croydon to mark the crash.
+2016-11-10 - The driver of the tram was arrested on suspicion of manslaughter.
+2016-11-15 - A statement was released by the family of one of the victims, Philip Logan.
+2016-11-</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>1. British Transport Police (BTP) - a police force responsible for policing the rail network in Great Britain, including light rail systems such as trams.
+2. Donald Collett, Philip Logan, and Robert Huxley - three victims of the Croydon tram crash who have been named by police.
+3. Croydon tram crash - a tragic event that occurred on November 9th, 2022 in Croydon, England, where a tram derailed and caused the deaths of seven people.
+4. Dorota Rynkiewicz, Mark Smith, Phil Seary, and Dane Chinnery - four other victims of the Croydon tram crash who have been named by police.
+5. Philip Logan - a victim of the Croydon tram crash who was described as a "true family man."
+6. Robert Huxley - a victim of the Croydon tram crash who was from New Addington.
+7. British Transport Police 22 (BTP22) - the Twitter handle used by the British Transport Police to share updates and information about the Croydon tram crash investigation.
+8. Croydon tram - a</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>1. The Croydon tram crash occurred because the two-carriage tram derailed at a speed of 50mph on a bend that had a speed limit of 12mph.
+2. The tram driver was arrested on suspicion of manslaughter after it was suspected that he might have been using his phone or have "blacked out" during the incident.
+3. The investigation into the accident is being conducted by the Rail Accident Investigation Branch (RAIB).
+4. The bodies of the victims were removed from the site by cranes and the damaged tram carriages were taken away on flatbed lorries.
+5. Repair work on the track was started by rail workers.
+6. Sections of the derailed tram were craned on to flatbed lorries and taken away from the scene.
+7. Family and friends of the victims paid tribute to them by leaving flowers and messages at the site of the accident.</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>1. The Croydon tram crash occurred on Wednesday morning.
+2. A two-carriage tram derailed at a sharp curve near Sandilands tram stop, travelling at a significantly higher speed than permitted.
+3. The crash resulted in the death of seven people, including Donald Collett, Philip Logan, and Robert Huxley.
+4. The other victims who had been named earlier were Mark Smith, Dane Chinnery, Phil Seary, and Dorota Rynkiewicz.
+5. The damaged tram cars were craned onto flatbed lorries on Saturday morning for removal from the scene.
+6. The Rail Accident Investigation Branch (RAIB) continues its inquiry into the cause of the accident.
+7. Friends and family of some of the victims marched to the site of the crash on Saturday to pay tribute.
+8. A group of up to 100 people gathered to remember the victims and leave floral tributes.
+9. One of the victims, Mark Smith, was due to get married next year.
+10. The driver of the tram has been arrested on suspicion of mansla</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Speaking from the Oval Office, Nov. 10, President Obama said he was "very encouraged" following a meeting with President-elect Donald Trump. Trump said the meeting lasted longer than expected and easily could have gone longer. (The Washington Post) President-elect Donald Trump and President Obama met for the first time Thursday and pledged to work together, starting the whirlwind transition that will unfold over the next 10 weeks until Trump is sworn into office Jan. 20. Trump later met with House Speaker Paul D. Ryan (R-Wis.) at the Capitol and said they also would work together -- but on Republican goals that are opposed by Obama and his fellow Democrats. "We're going to lower taxes," Trump told reporters, with Ryan seated by his side. "We're going to fix health care and make it affordable and better." He appeared to be referring to a plan to lower taxes that heavily benefits top earners and to the GOP's aim of repealing the Affordable Care Act, Obama's signature domestic policy achievement. Following his meeting with Ryan, Trump conferred with Senate Majority Leader Mitch McConnell (R) in the Kentucky senator's Capitol office. An hour and a half after Trump entered the White House through the South Lawn entrance -- avoiding news cameras and the president's staff -- a group of reporters was ushered into the Oval Office, where the president and president-elect were seated in the high-backed armchairs at the end of the room. In a sign of how tensions between the two politicians have not disappeared in the immediate aftermath of the election, the White House did not arrange for the traditional photo-op between the current first couple and the incoming one, a custom that George W. Bush and his wife Laura observed when the Obamas visited the White House in 2008. Melania Trump met separately with Michelle Obama. [Trump maps out a new administration to bring a seismic shift to Washington] Still, Trump told reporters Thursday that he expects to work closely with Obama now and in the future to seek his advice in guiding the country. He noted that a session that was supposed to last 10 to 15 minutes went on for an hour and a half. "As far as I'm concerned, it could have lasted a lot longer," Trump said. "We discussed a lot of different situations, some wonderful and some difficulties. I very much look forward to dealing with the president in the future, including counsel." "So Mr. President, it was a great honor being with you, and I look forward to being with you many, many more times in the future," he added, calling Obama "a very good man." 1 of 22 Full Screen Autoplay Close Skip Ad x What President-elect Donald Trump did on his trip to Washington View Photos Trump arrives at the White House for a meeting with Obama and on Capitol Hill to meet with Republican congressional leaders. Caption Trump arrives at the White House for a meeting with Obama and on Capitol Hill to meet with Republican congressional leaders. Nov. 10, 2016 President Obama talks with President-elect Donald Trump in the Oval Office of the White House in Washington. Jabin Botsford/The Washington Post Buy Photo Wait 1 second to continue. Obama, for his part, said, he was encouraged by "the interest in President-elect Trump's wanting to work with my team around many of the issues that this great country faces. And I believe that it is important for all of us, regardless of party and regardless of political preferences, to now come together, work together, to deal with the many challenges that we face." The president said that the men's two wives had enjoyed spending time together Thursday morning. "We want to make sure they feel welcome as they prepare to make this transition," Obama said. "Most of all, I want to emphasize to you, Mr. President-elect, that we now are going to want to do everything we can to help you succeed -- because if you succeed, then the country succeeds." [Trump's victory exposes Obama's inability to connect with white working class] Later, Trump and his wife, along with Vice President-elect Mike Pence, met with Ryan at the Capitol, where Trump pledged to work closely with Republican congressional leaders. Ryan ushered Trump out onto the Speaker's Balcony and gestured toward the Washington skyline and the monuments west of the Capitol. He pointed to an inaugural platform being built on the Capitol grounds, appearing to show Trump where he would be taking the oath of office as president. McConnell joined Trump and his entourage on a walking tour through part of the building. At the White House, first lady Michelle Obama and Melania Trump met for tea in the private residence and took a tour that included stepping onto Truman Balcony, as well as a tour of the State Floor with the White House curator. They talked about raising children in the White House, and then they visited the Oval Office to meet the president and president-elect. As the two leaders met, White House Chief of Staff Denis McDonough gave a tour to Trump's son-in-law, Jared Kushner, and other aides, notably Dan Scavino, across the edge of the Rose Garden. Afterward McDonough led Kushner on a walk down the South Lawn for nearly 20 minutes, at which point the two men rejoined Trump's senior staff and reentered the White House. During Obama and Trump's press availability, Kushner snapped photos with his iPhone. A slew of journalists, including international reporters, milled about on the driveway leading to the West Wing ahead of Trump's arrival. Some did live updates to their networks. Across West Executive Drive, dozens of White House staffers gathered on a steps in hopes of a glimpse of the president-elect. This is the scene on the West Wing driveway right now. pic.twitter.com/KoLxqek8qo -- David Nakamura (@DavidNakamura) November 10, 2016 Obama has pledged his administration's full cooperation with Trump's transition team, citing the close working relationship he enjoyed with President George W. Bush during their transfer of power eight years ago. The White House said that Pence met with Vice President Biden in the afternoon. "I have instructed my team to follow the example that President Bush's team set eight years ago and work as hard as we can to make sure that this is a successful transition for the president-elect," Obama said in the Rose Garden on Wednesday. The president said he called to congratulate Trump early Wednesday morning after news networks had formally announced Trump as the winner over Democratic nominee Hillary Clinton.' White House press secretary Josh Earnest told reporters after the meeting that the two men did not try to resolve all of their differences, but he said it was "a little less awkward" than reporters might have anticipated. Obama and Trump met privately without any other staff in the room. A large part of the Oval Office session was devoted to talking about how to staff and organize the White House. "That's complicated business," Earnest said, noting that presidents have to deal with multiple challenges and crises at the same time. It is "something President Obama has thought about extensively over the past eight years." Obama had denounced Trump as "temperamentally unfit" for the White House during a long and brutal campaign. But he said that "we are now all rooting for his success in uniting and leading the country. The peaceful transition of power is one of the hallmarks of our democracy. And over the next few months, we are going to show that to the world." Trump, and Clinton, already had been receiving national-security briefings as the nominees of the two major political parties. The White House said Thursday that Obama has convened a coordinating council to facilitate a smooth transition, including providing briefings from federal agencies to Trump's transition team, headed by New Jersey Gov. Chris Christie (R). Officials from the Trump transition team are starting to set up shop in agencies across the federal government, where they can consult with top Obama officials as they assemble their staffs. The current White House has already begun to transfer a massive amount of information to the National Archives and Records Administration: so far it has sent 283 million files, comprising 122,000 gigabytes of data. In an interview Wednesday, White House communications director Jennifer Psaki said the president has talked privately with his staff, as well as publicly, about putting institutional interests ahead of political ones. Referring to the speeches Obama delivered upon winning the presidency and at his first inaugural, she said: "He reflects a lot about the cog in the wheel that you are as president. He was taking the baton, he's handing it off. But I think it's a recognition that it's bigger than individual aspirations and it's bigger than yourself, and bigger than anything that you've accomplished. Because we as a country need to be stable, need to have continuity." In the wake of protests over Trump's win, Earnest said that while the president believes the protesters have a right to express their opinions, his message to them is that "we're Americans and patriots first" and that an orderly transfer of power ranks as a top White House priority. Ohio Gov. John Kasich (R), who ran unsuccessfully in the GOP presidential primary and harshly criticized Trump, was at the White House on Thursday to attend Obama's ceremony for the NBA champion Cleveland Cavaliers. Speaking to reporters outside the West Wing, Kasich said he saw people protesting Trump's election as he entered the White House gates, and he called for unity. "I just want to remind everyone in our country that the office of the presidency needs to be respected," he said. "Today, I said my prayers on the plane for the success of Donald Trump. And I think as Americans, we all need to come together." There is long-standing bad blood between Trump and Obama, after the New York businessman led a public campaign to try to force the president to disclose his long-form birth certificate in 2011 over unfounded questions from some conservatives who thought the president was not born in the United States. As a candidate, Donald Trump vowed to dismantle some of President Obama's key achievements. Washington Post White House reporter David Nakamura breaks down what the Obama administration is worried about going forward. (Sarah Parnass/The Washington Post) During the White House Correspondents' Association dinner that year, Obama lit into Trump, mocking him before a ballroom of 2,000 guests and on live television. During the campaign, Trump promised to repeal the president's signature health-care law and overturn many of his executive actions. Obama said Trump was not to be trusted with the nation's nuclear codes and represented an existential threat to democracy. Obama sought to play down their differences and said Trump's victory speech was magnanimous and set the right tone to help try to heal the nation's political divisions that were exposed and inflamed over the past 15 months. "They do not have an extensive personal relationship," Earnest said Wednesday, drawing laughs from reporters. "This is not a situation where they've had many conversations or played golf together or any of that business. So I guess that will be among the many, many, many reasons that tomorrow's meeting will be rather interesting." After his meeting with Trump, Obama welcomed another high-profile visitor with his own large media contingent: LeBron James and the NBA champion Cleveland Cavaliers.</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>meets with Obama; pledged to work together</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>at the White House</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Nov. 10; Thursday </t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Donald Trump; President Obama</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr"/>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>encouraged</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>1. Trump and Obama meet for the first time at the Oval Office.
+2. Trump and Ryan meet at the Capitol and discuss Republican goals.
+3. Trump meets with McConnell at the Capitol.
+4. Melania Trump meets with Michelle Obama.
+5. Obama and Trump discuss the transition process and how to staff the White House.
+6. Trump's team begins to set up shop in federal agencies.
+7. Protests against Trump's victory take place.
+8. Obama urges unity and respect for the office of the presidency.
+9. Trump and Obama discuss the repeal of Obama's healthcare law and executive actions.
+10. Obama and Trump's long-standing bad blood is briefly mentioned.
+11. Obama and Trump discuss the importance of a peaceful transition of power.
+12. Kasich meets with Obama and urges Americans to come together.
+13. Trump and Obama's dissimilarities are acknowledged.
+14. Obama awards the Cleveland Cavaliers with the NBA championship trophy.</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>[United States, District of Columbia, Washington, D.C.]
+[United States, Ohio, Cleveland]</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>2016-11-10 (Oval Office meeting)
+2016-11-10 (meeting with House Speaker Paul D. Ryan)
+2016-11-10 (meeting with Senate Majority Leader Mitch McConnell)
+2016-11-10 (Trump and Obama discussing staffing and organizing the White House)
+2016-11-09 (Trump wins the election)
+2016-11-08 (Obama and Clinton have their last debate)
+2016-11-07 (Obama calls to congratulate Trump)
+2016-09-26 (Trump accepts the Republican nomination)
+2016-07-21 (Trump and Obama meet at the White House)
+2016-07-15 (Clinton accepts the Democratic nomination)
+2016-07-05 (Obama meets with both Clinton and Trump)</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">President Barack Obama
+President-elect Donald Trump
+House Speaker Paul D. Ryan (R-Wis.)
+Vice President Joe Biden
+Melania Trump
+Michelle Obama
+Vice President-elect Mike Pence
+Senate Majority Leader Mitch McConnell (R)
+White House Chief of Staff Denis McDonough
+Jared Kushner
+Dan Scavino
+David Nakamura
+Sarah Parnass
+What are the main events described in the text? List and enumerate (in English)::
+</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1. The meeting between President Obama and President-elect Donald Trump occurred because Trump won the 2016 presidential election, making him the next President of the United States. It was important for both leaders to meet and discuss the transition of power.
+2. Trump and House Speaker Paul Ryan met to discuss their shared goals, which include lowering taxes and repealing the Affordable Care Act. They also discussed other Republican priorities.
+3. Trump met with Senate Majority Leader Mitch McConnell to discuss their agenda and work together on issues they support.
+4. The White House arranged for Obama and Ryan to meet separately to discuss the transition of power and coordinate on areas of agreement.
+5. Melania Trump met with Michelle Obama to discuss the transition and their roles as First Ladies.
+6. President Obama and the Trump team held a meeting to discuss the transition process and ensure a smooth handover of power.
+7. President Obama and the Trump team discussed staffing and organizing the White House, as part of the transition process.
+8. Obama and Trump had a private meeting to discuss their differences and find areas of agreement for the good of the country.
+</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>1. Donald Trump and President Obama met for the first time. They discussed a lot of different situations and topics, including health care and taxes. The meeting lasted longer than expected and could have gone longer.
+2. After the meeting with President Obama, Trump met with House Speaker Paul D. Ryan (R-Wis.) at the Capitol. They discussed working together on Republican goals, specifically focusing on repealing the Affordable Care Act and lowering taxes, which heavily benefit top earners.
+3. Trump also met with Senate Majority Leader Mitch McConnell (R) in the Kentucky senator's Capitol office.
+4. Melania Trump met separately with Michelle Obama.
+5. President-elect Trump and his team began transitioning into their new roles and working with federal agencies to prepare for the upcoming inauguration.
+6. The White House hosted a meeting between Donald Trump and Paul Ryan, which was followed by a press conference where both men spoke about their plans and intentions for the future.
+7. The White House press secretary, Josh Earnest, addressed the media and discussed the meeting between President Obama and Donald Trump, noting that the two</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
           <t>Skip Ad Ad Loading... x Embed x Share Toblerone is facing a mountain of criticism for changing the shape of its famous triangular candy bars in British stores, a move it blames on rising costs. USA TODAY Toblerone chocolate bars come in a variety of sizes, but recently changed the shape of two of its smaller bars sold in the UK. (Photo: Martin Ruetschi, AP) The UK has a chocolate bar crisis on its hands: the beloved Swiss chocolate bar is unrecognizable. Toblerone, the classic chocolate bar with almond-and-honey-filled triangle chunks, recently lost weight. In two sizes, the triangles shrunk, leaving wider gaps of chocolate. Toblerone can you tell me what this is all about... looks like there's half a bar missing! pic.twitter.com/C2VD3DjppE -- Alana Cartwright (@AlanaCartwrigh3) October 29, 2016  @HelenRyles Hi Helen, yes this is just our smaller bar. -- Toblerone (@Toblerone) October 31, 2016  The 400-gram bar was reduced to a 360-gram bar and the 170-gram was reduced to 150 grams. "Like many other companies, we are experiencing higher costs for numerous ingredients ... we have had to reduce the weight of just two of our bars in the UK," the company said on Facebook. People aren't happy about the change. The new #Toblerone. Wrong on so many levels. It now looks like a bicycle stand.#WeWantOurTobleroneBack. pic.twitter.com/C71KeNUWF1 -- James Melville (@JamesMelville) November 8, 2016  So unhappy, in fact, it's outpacing U.S. Election Day news. I'm so happy that readers of BBC News have got their priorities right. #Toblerone#Election2016pic.twitter.com/eeAlvoTqY6 -- David Wriglesworth (@Wriggy) November 8, 2016 It could be the end of the world as we know it. So what are the good folk of Britain talking about? Toblerone. pic.twitter.com/i8ryxmHc5c -- Julia Hartley-Brewer (@JuliaHB1) November 8, 2016 Some blame Brexit. Straight up the worst thing about brexit is Toblerone down sizing -- Alex Littlewood (@Alex_JL29) November 8, 2016 #toblerone#brexit I told you that leaving the EU would have serious consequences. Now I' m really upset. pic.twitter.com/w81cWYpNl4 -- Mark Greenwood (@markcjgreenwood) November 8, 2016 The company denies the change is tied to Brexit, a Mondelez spokeswoman told the BBC. The only bars affected are sold in the UK. Follow Ashley May on Twitter: @ashleymaytweets Read or Share this story: http://usat.ly/2fcLZ18</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
+      <c r="B5" t="inlineStr">
         <is>
           <t>outraged over Toblerone chocolate</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
+      <c r="C5" t="inlineStr">
         <is>
           <t>in British stores; UK</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
+      <c r="D5" t="inlineStr">
         <is>
           <t>November 8, 2016</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr">
+      <c r="E5" t="inlineStr">
         <is>
           <t>UK; Toblerone</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr">
+      <c r="F5" t="inlineStr">
         <is>
           <t>changing the shape of its famous triangular candy bars</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr">
+      <c r="G5" t="inlineStr">
         <is>
           <t>changed the shape</t>
         </is>
       </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>1. Toblerone chocolate bars change their shape in British stores due to rising costs.
-2. The company explains that the change affects only two of their bars sold in the UK.
-3. Consumers express their disappointment and unhappiness with the new shape of Toblerone chocolate bars.
-4. Some people tie the change to the Brexit decision, but the company denies any connection.</t>
-        </is>
-      </c>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> [Switzerland,United Kingdom]</t>
-        </is>
-      </c>
-      <c r="J2" t="inlineStr">
-        <is>
-          <t>The events described in the text occurred on or around:
-1. 2016-10-29 - Toblerone changes shape in British stores
-2. 2016-11-08 - People start complaining about the change</t>
-        </is>
-      </c>
-      <c r="K2" t="inlineStr">
-        <is>
-          <t>1. Toblerone - a Swiss chocolate bar company
-2. Mondelez - the company that owns Toblerone
-3. UK consumers - people who live in the United Kingdom and have purchased Toblerone chocolate bars
-4. Helen Ryles and Alana Cartwright - Twitter users who have expressed their dissatisfaction with the change in Toblerone's shape
-5. James Melville, David Wriglesworth, Julia Hartley-Brewer, Alex Littlewood, and Mark Greenwood - Twitter users who have shared their opinions about the situation
-6. BBC News - the British Broadcasting Corporation, a news organization that has covered the story</t>
-        </is>
-      </c>
-      <c r="L2" t="inlineStr">
-        <is>
-          <t>1. The Toblerone chocolate bars changed shape in the UK due to rising costs of ingredients.
-2. The change in shape affected two sizes of Toblerone bars: the 400-gram bar was reduced to a 360-gram bar and the 170-gram was reduced to 150 grams.
-3. The company, Mondelēz, blamed higher costs for numerous ingredients as the reason for the change.
-4. The new shape of the Toblerone bars sparked outrage among consumers, leading to widespread criticism and negative reactions on social media.
-5. Some people attributed the change to the economic impact of Brexit, while the company denied any connection.</t>
-        </is>
-      </c>
-      <c r="M2" t="inlineStr">
-        <is>
-          <t>1. Toblerone, a Swiss chocolate brand, changed the shape of two of its smaller bars sold in the UK.
-2. The change resulted in wider gaps between the triangular chunks of chocolate and almonds.
-3. The company cited rising costs of ingredients and blamed it on "higher costs for numerous ingredients."
-4. The reduced sizes affected both the 400-gram and 170-gram bars, which were reduced to 360 grams and 150 grams respectively.
-5. The public expressed their dissatisfaction with the change, with some even going as far as to say it was worse than the U.S. election news.
-6. Some people attributed the change to Brexit, while the company denied any connection.
-7. The change only affected UK stores, and did not impact other markets or product sizes.</t>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>1. Toblerone changes the shape of two of its smaller chocolate bars sold in the UK.
+2. The company explains that the change is due to rising costs for ingredients.
+3. The public reacts negatively to the new shape of the chocolate bars.
+4. Criticism of the change becomes widespread on social media and news outlets.
+5. Some people blame Brexit for the change, but the company denies any connection.</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> The events described in the text occurred in the United Kingdom (UK).</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>The text does not provide specific dates.</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>1. Toblerone - Swiss chocolate brand
+2. Mondelez - parent company of Toblerone
+3. UK consumers - people affected by the change in Toblerone's chocolate bar sizes
+4. Alana Cartwright - Twitter user who expressed dissatisfaction with the change
+5. Helen Ryles - Twitter user who asked Toblerone about the change
+6. BBC News - British news organization that reported on the story
+7. James Melville - Twitter user who expressed discontent with the change
+8. David Wriglesworth - Twitter user who compared the coverage of Toblerone and U.S. Election Day news
+9. Julia Hartley-Brewer - Twitter user who commented on the news coverage
+10. Alex Littlewood - Twitter user who blamed Brexit for the Toblerone change
+11. Mark Greenwood - Twitter user who made a joke about Brexit and the Toblerone change
+12. Ashley May - USA TODAY reporter who wrote the article</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>1. Toblerone changed the shape of its smaller bars sold in the UK due to rising costs of ingredients.
+2. The UK population is unhappy with the change and has expressed their dissatisfaction on social media and in the news.
+3. The Toblerone controversy has become a topic of discussion and humor among the public, even overshadowing some important events like the US Election Day news.
+4. Some people blame Brexit for the Toblerone shape change, claiming that it is a result of the economic instability caused by the UK leaving the European Union. However, the company denies any connection between the two events.</t>
+        </is>
+      </c>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>1. Toblerone, a Swiss chocolate bar company, faced rising costs for ingredients.
+2. As a result, they had to reduce the weight of two of their bars sold in the UK: the 400-gram bar was reduced to 360 grams, and the 170-gram bar was reduced to 150 grams.
+3. The company explained this decision by saying that they were not alone in experiencing higher costs for ingredients.
+4. The change in the chocolate bars' weight and shape upset customers in the UK.
+5. People reacted strongly on social media, expressing their displeasure and disappointment with the new Toblerone sizes.
+6. Some blamed the decision on Brexit, while the company denied any connection between the two events.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>The death toll from a powerful Taliban truck bombing at the German consulate in Afghanistan's Mazar-i-Sharif city rose to at least six Friday, with more than 100 others wounded in a major militant assault. The Taliban said the bombing late Thursday, which tore a massive crater in the road and overturned cars, was a "revenge attack" for US air strikes this month in the volatile province of Kunduz that left 32 civilians dead. The explosion, followed by sporadic gunfire, reverberated across the usually tranquil northern city, smashing windows of nearby shops and leaving terrified local residents fleeing for cover. "The suicide attacker rammed his explosives-laden car into the wall of the German consulate," local police chief Sayed Kamal Sadat told AFP. All German staff from the consulate were unharmed, according to the foreign ministry in Berlin.</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>attacks German consulate; truck bombing</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>northern Afghan city of Mazar-i-Sharif</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>late Thursday</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Taliban</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>revenge attack</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>rammed his explosives-laden; rammed</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 1. A powerful Taliban truck bombing at the German consulate in Afghanistan's Mazar-i-Sharif city
+2. The death toll rose to at least six people, with more than 100 others wounded
+3. The Taliban claimed responsibility, calling it a "revenge attack" for US air strikes in Kunduz that left 32 civilians dead
+4. The explosion occurred late Thursday, followed by sporadic gunfire
+5. The blast smashed windows of nearby shops and sent terrified locals fleeing for cover
+6. The suicide attacker rammed an explosives-laden car into the wall of the German consulate
+7. All German staff at the consulate were unharmed, according to the foreign ministry in Berlin</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> [Afghanistan,Balkh,Mazar-i-Sharif]</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> The events described in the text occurred on [2016-11-10].
+List of events:
+1. The Taliban truck bombing at the German consulate in Mazar-i-Sharif city, Afghanistan.
+2. The death toll from the Taliban attack rose to at least six people.
+3. More than 100 others were wounded in the major militant assault.
+4. The Taliban claimed responsibility for the attack, calling it a "revenge attack" for US air strikes in Kunduz that killed 32 civilians.
+5. The explosion occurred late Thursday, followed by sporadic gunfire.
+6. The suicide attacker rammed his explosives-laden car into the wall of the German consulate.
+7. Local police reported that all German staff from the consulate were unharmed.
+8. The foreign ministry in Berlin confirmed that all German staff were safe.
+9. The explosion smashed windows of nearby shops and terrified local residents fled for cover.
+10. The aftermath of the attack left a massive crater in</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 1. Taliban - an Islamic fundamentalist political movement and military organization in Afghanistan. They claim responsibility for the attack.
+2. German consulate - the diplomatic mission of Germany in Afghanistan.
+3. Afghanistan - the country where the consulate is located.
+4. Mazar-i-Sharif city - the location of the German consulate where the attack took place.
+5. Kunduz province - the province where US air strikes occurred, which the Taliban claimed as the reason for their attack.
+6. US - the United States, which carried out the air strikes in Kunduz.
+7. Local police - the law enforcement agency responsible for maintaining peace and order in Mazar-i-Sharif city.
+8. Sayed Kamal Sadat - the local police chief who provided information about the attack.
+9. Foreign ministry in Berlin - the diplomatic body of Germany responsible for international relations.
+10. German staff - the individuals working at the German consulate in Mazar-i-Sharif city.</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>1. The Taliban carried out a truck bombing at the German consulate in Mazar-i-Sharif, Afghanistan, as a "revenge attack" for US air strikes in the province of Kunduz that killed 32 civilians this month. The Taliban claimed responsibility for the attack.
+2. The suicide bomber drove an explosives-laden car into the wall of the German consulate, causing extensive damage and killing at least six people, with over 100 others injured.
+3. The explosion and subsequent gunfire terrified local residents, who fled the area and sought cover.
+4. The German foreign ministry reported that all German staff from the consulate were unharmed in the attack.
+Note: The events occurred because of the Taliban's desire for retaliation against the US air strikes in Kunduz and their targeting of the German consulate in Mazar-i-Sharif.</t>
+        </is>
+      </c>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 1. A powerful Taliban truck bombing took place at the German consulate in Afghanistan's Mazar-i-Sharif city.
+2. The explosion occurred late Thursday, leaving a massive crater in the road and overturning cars.
+3. The bombing was a "revenge attack" for US air strikes this month in the volatile province of Kunduz that left 32 civilians dead.
+4. The explosion was followed by sporadic gunfire.
+5. The attacker rammed an explosives-laden car into the wall of the German consulate.
+6. The suicide attacker was part of the Taliban.
+7. The police chief, Sayed Kamal Sadat, reported the incident.
+8. The foreign ministry in Berlin confirmed that all German staff from the consulate were unharmed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Max Verstappen produced a flourish to finish third at the Brazil Grand Prix Christian Horner, the Red Bull team principal, has described Max Verstappen's incredible performance in Sunday's Brazilian Grand Prix as one of the best he has ever witnessed in Formula One. Verstappen overtook half the field in the closing stages of the rain-soaked race to claim the final spot on the podium behind race winner Lewis Hamilton and Nico Rosberg. The 19-year-old Dutchman, who had been running second only to Hamilton following a brilliant move around the outside of championship leader Rosberg, dropped way down the order after his team opted to pit him for the intermediate tyre, only to call him in again for the extreme wet option. Max Verstappen produced an incredible display at the Brazil Grand Prix at Interlagos Red Bull chief Christian Horner said Verstappen's race was one of the finest drives he has seen But the teenager overtook 13 cars - including that of his team-mate Daniel Ricciardo and Sebastian Vettel, the four-time world champion whom he left trailing on the grass - to claw his way on to the podium in one of the most impressive displays in recent grand prix memory. 'His recovery was amazing, and that was one of the best drives I've seen in Formula One,' a jubilant Horner said on Sunday night. 'We gave him a huge amount to do and the way he drove those last 15 laps was unbelievable. The young Dutchman overcame adverse weather to produce a masterclass at Interlagos In the pits, the Red Bull team went wild as Verstappen secured a podium finish 'Max was in a league of his own today, and what we witnessed was something very, very special.' While Hamilton sauntered to victory in the treacherous conditions to keep his championship hopes alive, Verstappen stole the show with his virtuoso display in a race filled with drama. At the first re-start Verstappen immediately passed Kimi Raikkonen, the 2007 world champion, with a banzai move at turn one, before he delivered the same treatment around the outside of Rosberg at turn three later in the race. He also survived a hairy moment as he lost control of his Red Bull at close to 180mph when he entered the pit straight. Incredibly, the teenager managed to avoid any contact with the barrier, and remained ahead of Rosberg, too. 'The heartbeat went a bit higher there,' he said coolly over the team radio. Verstappen earned his spot in the limelight after overtaking half the field in the closing stages Spray and standing water meant visibility was severely limited... but it didn't stop Verstappen Verstappen was on course to finish second, and possibly challenge Hamilton for the win, but Red Bull's gamble to put him on the intermediate tyre backfired. 'Win? Maybe not, but I think second was definitely possible,' Verstappen said. 'I think we were in quite a safe position in second but sometimes you have to gamble to try and win the race.</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>amazes Red Bull principal Christian Horner; has described Max Verstappen's performance</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Brazil; Brazilian Grand Prix; Interlagos</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Sunday</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>Max Verstappen; Christian Horner</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>overtook half the field; incredible performance; produced a flourish to finish third</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>finish third; witnessed</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>1. Max Verstappen's impressive performance at the Brazilian Grand Prix
+2. Red Bull's decision to pit Verstappen for the intermediate tyre
+3. Verstappen's overtaking maneuvers, including passing Hamilton's teammate and championship leader Nico Rosberg
+4. Verstappen's recovery after dropping down the order due to pit strategy
+5. Christian Horner's praise for Verstappen's drive as one of the best he's seen in Formula One
+6. Verstappen's near-miss with Kimi Raikkonen and Nico Rosberg during overtaking attempts
+7. Verstappen's hair-raising moment when he lost control of his car at close to 180mph on the pit straight
+8. Verstappen's ability to avoid contact with the barrier and maintain position in the race
+9. The drama and chaos caused by adverse weather conditions during the race
+10. The impact of Red Bull's pit strategy on Verstappen's final position in the race</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> Brazil, São Paulo, Interlagos</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> The events described in the text occurred on [2016-11-13].
+Events:
+1. Max Verstappen's incredible performance at the Brazilian Grand Prix
+2. Red Bull team principal Christian Horner describing it as one of the best he has ever witnessed in Formula One
+3. Verstappen overtaking half the field in the closing stages of the race to finish third
+4. Red Bull team's gamble to put him on the intermediate tyre backfiring
+5. Max Verstappen's overtaking moves on Kimi Raikkonen, Sebastian Vettel, and Nico Rosberg
+6. Verstappen surviving a hairy moment at close to 180mph without hitting the barrier
+7. Red Bull chief Christian Horner calling it one of the finest drives he has seen in Formula One
+8. Lewis Hamilton winning the race, keeping his championship hopes alive
+9. The race filled with drama due to adverse weather conditions</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>1. Max Verstappen: A 19-year-old Dutch Formula One driver for Red Bull Racing.
+2. Christian Horner: The team principal of Red Bull Racing.
+3. Daniel Ricciardo: Another Red Bull Racing driver.
+4. Sebastian Vettel: A four-time World Champion Formula One driver.
+5. Lewis Hamilton: The race winner of the Brazilian Grand Prix.
+6. Nico Rosberg: The championship leader and runner-up of the Brazilian Grand Prix.
+7. Red Bull: Max Verstappen's racing team.
+8. Kimi Raikkonen: A Finnish Formula One driver for Ferrari.
+9. Red Bull Racing: Max Verstappen's team.
+10. Interlagos: The racetrack where the Brazilian Grand Prix took place.
+What is the main event or topic discussed in the text?
+The main event discussed in the text is Max Verstappen's outstanding performance during the Brazilian Grand Prix at Interlagos, where he managed to overtake half the field in the closing stages of the race, despite facing adverse weather conditions and making some questionable pit stops.</t>
+        </is>
+      </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>1. Max Verstappen's incredible performance: This event occurred because of his outstanding driving skills and strategy during the Brazilian Grand Prix. He overtook half the field in the closing stages, displaying incredible speed and precision.
+2. Red Bull's pit stop decision: This event occurred due to Red Bull's decision to pit Verstappen for the intermediate tyre, which didn't work out as planned. The team had to call him in again for the extreme wet option.
+3. Difficult weather conditions: The treacherous weather, including rain, played a significant role in the events that unfolded during the race. This affected visibility and grip, making driving even more challenging for the drivers.
+4. Dramatic situations: The race was filled with dramatic moments, such as Verstappen's move around the outside of other drivers and his near-miss with the barrier. These situations added to the excitement and unpredictability of the event.
+5. Title race implications: The race also had significant implications for the championship, as Hamilton's victory kept his championship hopes alive. This added an extra layer of pressure and significance to Verstappen's performance.</t>
+        </is>
+      </c>
+      <c r="M7" t="inlineStr">
+        <is>
+          <t>1. Verstappen's team, Red Bull, pitted him for the intermediate tyre, hoping to gain an advantage in the rainy conditions.
+2. The team then called Verstappen in again for the extreme wet option, but he was running behind his teammate Daniel Ricciardo at the time.
+3. In the treacherous conditions, Verstappen made a brilliant move around the outside of championship leader Nico Rosberg at turn three.
+4. As the race progressed, visibility became increasingly poor due to spray and standing water on the track.
+5. Near the end of the race, Verstappen began to lose places and dropped down the order, eventually finding himself way behind Sebastian Vettel and other top drivers.
+6. Despite being in a difficult position, Verstappen put on an incredible display of driving skill, overtaking 13 cars, including Vettel, to claw his way back onto the podium in third place.
+7. This impressive comeback drive was praised by Red Bull team principal Christian Horner as one of the best he had ever witnessed in Formula One.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Toblerone has come under fire after it increased the space between the distinctive triangles of its bars. Mondelez International, the company which makes the product, said the change was made due to price rises in recent months, however consumers called the move "obscene". "Like many other companies, we are experiencing higher costs for numerous ingredients. We carry these costs for as long as possible, but to ensure Toblerone remains on-shelf, is affordable and retains the triangular shape, we have had to reduce the weight of just two of our bars in the UK, from the wider range of available Toblerone products," the company wrote on its Facebook page. However many questioned the necessity of the move, commenting that Toblerone does not constitute an everyday purchase and therefore customers would be able to absorb a price rise. Others called the change "underhanded" accusing the company of masking the fact the bar is smaller. The change has seen the 400g bars reduced to 360g and the 170g bars to 150g, with the size of the packaging remaining the same. And they've changed the Toblerone, quite obviously so you less triangles in a row. Typical cost cutting measure. -- Angela Night (@Angelheartnight) November 8, 2016  "Fair enough reducing the weight of the bar, but why the big gap in between segments? Looks stupid, could have just made the bar shorter and kept the original design," Lee Yarker wrote on Facebook. My god, the Toblerone change is obscene. #mindthegap pic.twitter.com/VnXFaiFAml -- Josh Barrie (@joshbythesea) November 8, 2016 Mondelez International is not the first company to announce price rises as a result of the falling pound. Madness. Why mess with the single distinctive feature of the product? Who monitors price of a Toblerone anyway, hardly a household staple? https://t.co/DovjffjOJP -- Chris Duncan (@chrisduncania) November 8, 2016 In October, Tesco and Unilever clashed after the company said it would raise prices of its key products to compensate for the diminishing value of British currency. The Independent has contacted Mondelez International for comment.</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>sparks outrage; has come under fire</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>UK</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>November 8, 2016</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>Toblerone; Mondelez International</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>changing iconic shape; increased the space between the distinctive triangles of its bars; due to price rises</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>increased the space</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>1. Toblerone, a chocolate bar manufactured by Mondelez International, increased the space between its distinctive triangles.
+2. Mondelez International explained the reason for the change as a result of price rises in recent months.
+3. Consumers reacted negatively to the change, calling it "obscene" and "underhanded."
+4. Many consumers questioned the necessity of the change, arguing that Toblerone is not an everyday purchase.
+5. The change affected the 400g and 170g bars, reducing their weight to 360g and 150g respectively, while keeping the size of the packaging the same.
+6. The company also reduced the number of triangles in a row in some of the bars.
+7. Social media users reacted to the news, expressing their disapproval and questioning the design change.
+8. The Toblerone controversy was placed in the context of other price increases in the UK market, such as those faced by Tesco and Unilever.</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> United Kingdom (UK)</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> - November 8, 2016: Mondelez International announced the change in Toblerone design and weight due to price rises.
+ - October, 2016: Clash between Tesco and Unilever over price increase of key products caused by falling pound value.
+ - [unspecified date]: The Independent contacted Mondelez International for comment.</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>1. Toblerone - a chocolate brand owned by Mondelez International
+2. Mondelez International - the company that manufactures Toblerone
+3. Consumers - individuals who purchase and use Toblerone
+4. Price rise - an increase in the cost of goods, in this case, Toblerone
+5. Facebook page - the official social media page of Toblerone's parent company
+6. Angela Night - a Twitter user who commented on the Toblerone change
+7. Lee Yarker - a Facebook user who criticized the design change of Toblerone
+8. Josh Barrie - a Twitter user who shared his opinion on the Toblerone change
+9. Chris Duncan - a Twitter user who commented on the Toblerone change and the overall situation
+10. Tesco - a British supermarket chain
+11. Unilever - a consumer goods company that clashed with Tesco over price increases in October</t>
+        </is>
+      </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>1. Toblerone's distinctive triangular shape has been altered due to rising production costs.
+2. Mondelez International, the company that makes Toblerone, claims that the change was made to maintain the product's affordability and retain its triangular shape.
+3. Consumers have criticized the move as "obscene" and "underhanded," questioning the necessity of the change and accusing the company of masking the fact that the bar is smaller.
+4. The change in design has led to a reduction in the weight of two Toblerone bar sizes: the 400g bars are now 360g, and the 170g bars are now 150g.
+5. The packaging size remains unchanged.
+6. The price of Toblerone has increased due to rising production costs, but the company has tried to absorb these costs for as long as possible.
+7. The falling value of the British pound following the Brexit vote has led to price increases across various consumer goods, including Toblerone, as companies like Mondelez International struggle to maintain profit margins.</t>
+        </is>
+      </c>
+      <c r="M8" t="inlineStr">
+        <is>
+          <t>1. Toblerone, a chocolate brand owned by Mondelez International, increased the space between the distinctive triangles of its bars.
+2. The company made this change due to price rises in recent months.
+3. Consumers reacted negatively to the change, calling it "obscene" and "underhanded."
+4. The change resulted in a reduction of the weight of two of the bars available in the UK, from 400g to 360g, and from 170g to 150g.
+5. The company defended the move by stating that they were experiencing higher costs for ingredients and trying to keep the product affordable.
+6. Some consumers questioned the necessity of the change, arguing that Toblerone is not an everyday purchase and price increases should be absorbed.
+7. Others accused the company of masking the fact that the bar was smaller by changing its design.
+8. The falling pound has led to price rises in various products, including Toblerone, which in turn has forced companies to make changes to their products and pricing strategies.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Driver is retiring at the end of the season bringing down the curtain on a wonderful career that has seen him become one of the most liked and popular in the sport Click to share on WhatsApp (Opens in new window) Click to share on Facebook (Opens in new window) Click to share on Twitter (Opens in new window) FELIPE MASSA didn't have the winning send off he would have liked in his last home Grand Prix after crashing in awful conditions. Massa's Williams car crashed in lap 48 as the Brazilian struggled to cope with the endless downpour on his home track of Interlagos. AP:Associated Press 5 Felipe Massa waves to the crowd of adoring fans after the race Getty Images 5 The Brazilian is retiring from F1 at the end of the season and raced for the last time at Interlagos Getty Images 5 Massa sits down whilst the race was suspended due to heavy rain Massa escaped the circuit and the weather to huge cheers from the crowd as it finally hit home that one of greats of F1 is about to retire. The Brazilian fought back tears as he was overwhelmed by the emotion coming from his home crowd. Massa said: "It's difficult to explain the feeling. To not manage to finish the race, for my fans, for Brazil. "This place is so special for me but God knows what to do. "It's so special from the people in Brazil, in the paddock, everyone that I work for. "I just say thank you very much. It's a real honour, a real pleasure. "It's difficult to explain. related articles Gunning for glory How can Nico Rosberg can be crowned as Formula One world champion this weekend? CHANGE OF GEAR Serena Williams and Lewis Hamilton cosy up and hold hands at Formula One Mexican Grand Prix 21 Pog Street Two-time Oscar Nominee Jonah Hill is spotted sporting a Paul Pogba top...but it's not a Red Devils shirt! Rich List Man Utd have the biggest wage bill in world football, with players on average of PS5.77m a year Gunned Down Alexis Sanchez just 2/1 to leave Arsenal and join Premier League rivals Manchester City "So special to see these guys [in the pit lane] going out just to see me passing after the crash. "Thank you very much. I will never forget this day. All these people, all you guys will be in my heart forever." "I didn't deserve so much like that. "I could have finished the race, but maybe it was better like that." Getty Images 5 Massa cries as he heads down the pit lane Getty Images 5 The Williams driver is given a guard of honour by his rival teams The pits were united in showing their appreciation as all the crews paid homage to a sporting great who has given everything to the sport he loves dearly. Massa was given a guard of honour as he walked to meet his wife Anna Raffaella and son Felipinho whom he hugged, kissed and sobbed. Lewis Hamilton eventually won a very dangerous Grand Prix that saw a number of cars aquaplaning across the track with the worry that life threatening accidents could be on the verge of unfolding if the weather was to continue to get worse. Fortunately there were no serious injuries amongst the crashes and the debris as the championship is still left hanging in the balance. The Portuguese national team looks good doing the latest craze</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>very emotional farewell after crashing</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Interlagos</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>end of the season; race in Brazil</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>FELIPE MASSA</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>last home race in Brazil; awful conditions</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr"/>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>1. Felipe Massa crashes in the last lap of his last home Grand Prix due to heavy rain.
+2. Massa is overwhelmed with emotions as he realizes this is his last race.
+3. The Brazilian thanks his fans, team, and everyone in the paddock for their support throughout his career.
+4. Massa is given a guard of honor by rival teams as he leaves the circuit.
+5. Lewis Hamilton wins a dangerous race amidst heavy rain and aquaplaning.
+6. The championship is left hanging in the balance.</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> Brazil, Sao Paulo, Interlagos</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>2016-11-13 - Felipe Massa's retirement announcement
+2016-11-13 - Felipe Massa's last home Grand Prix
+2016-11-13 - Felipe Massa's crash during the race
+2016-11-13 - Lewis Hamilton's win in the race
+2016-11-13 - End of the Brazilian Grand Prix</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>1. Felipe Massa - A former Formula One driver
+2. Interlagos - A race track in Brazil
+3. Williams - A Formula One team
+4. Fans - People who support Felipe Massa and were at the race
+5. Other drivers and teams - Competitors of Felipe Massa and Williams in the race
+6. Anna Raffaella and Felipinho - Felipe Massa's wife and son
+7. Lewis Hamilton - A Formula One driver
+8. Race organizers - People in charge of the race
+9. Weather - The condition that caused the accidents during the race
+10. Championship - The title of the highest-ranking driver or team in the sport</t>
+        </is>
+      </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>1. Felipe Massa crashed in his last home Grand Prix because he couldn't handle the heavy rain.
+2. The race was suspended due to the heavy rain, making it difficult for drivers to maintain control of their vehicles.
+3. Massa's retirement was celebrated by his adoring fans, with many of them coming out to see his last race.
+4. The pits and rival teams showed their appreciation for Massa's contributions to the sport by giving him a guard of honor and a warm sendoff.
+5. The championship is still undecided as the race was won by Lewis Hamilton, but the overall winner will be determined in the next race.</t>
+        </is>
+      </c>
+      <c r="M9" t="inlineStr">
+        <is>
+          <t>1. Felipe Massa, a popular and respected driver, announced his retirement from Formula One (F1) at the end of the season.
+2. His retirement was marked by his last home Grand Prix at Interlagos, where he raced for Williams.
+3. During the race, heavy rain caused poor visibility and made it difficult for drivers to maintain control of their cars.
+4. In lap 48, Massa's car crashed due to the poor weather conditions.
+5. The crowd, which was full of adoring fans, reacted with shock and dismay at the crash.
+6. Massa walked out of the car and the track, visibly emotional and overwhelmed by the support he received from his home crowd.
+7. Despite the crash, Massa was given a guard of honour by rival teams as he left the pit lane.
+8. The pits and pit crews paid tribute to Massa, showing their appreciation for his dedication and contribution to the sport.
+9. Lewis Hamilton won the race in dangerous conditions, with several other drivers also experiencing crashes or near-misses.
+10. The championship remains und</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Teenage Formula One star Max Verstappen showed nerves of steel as he somehow managed to avoid a serious accident despite spinning his car at 180mph in dangerous conditions at the Brazilian Grand Prix. Travelling flat out at the Interlagos circuit, Verstappen lost control as he clipped the curb on the entrance to the long home straight, spinning his car sideways and sliding dangerously down the track. But just as it looked as though he was going to smash the nose of his car into the metal side hoardings, which would likely have seen his car catapulted into the middle of the track and into the path of other cars, he was able to straighten up and regain control. Max Verstappen clipped the curb on his way up the hill towards the home straight in Brazil That caused Verstappen to lose control of his car as his back end slid round as he spun With the nose of his Red Bull car pointing towards the wall, Verstappen slid down the track Verstappen produced an incredible display to finish third at the Brazilian Grand Prix Immediately after the incident a member of Verstappen's Red Bull pit crew calmly said 'well held Max, well held' on the team radio before the driver himself joked 'my heartbeat went a little higher there.' While many would have been shaken by such a high-speed incident, Verstappen showed maturity beyond his years as he recovered to eventually secure third place in the Grand Prix, behind Lewis Hamilton and Nico Rosberg. Verstappen is one of the hottest teenage talents F1 has ever seen and in his two seasons in the sport has thrilled and frustrated in equal measure, with an aggressive driving style which has split opinion both in the pits and in the stands. But the 19-year-old gained universal praise for the way he avoided a serious accident in hazardous conditions in Brazil, during a race in which a number of spectacular crashes caused major delays as drivers struggled to cope with the wet weather. The back of Verstappen's car slid out as the camera cut to show the view of the home straight That left Verstappen in a vulnerable position, with his car side on and facing the barrier But as he slid further and further down the track, Verstappen was able to straighten up Miraculously he was able to drive away from the incident without hitting the wall of the track The young Dutchman overcame adverse weather to produce a masterclass at Interlagos WHO IS MAX VERSTAPPEN? - Max Verstappen was born on September 30, 1997 in Belgium - The teenager is the son of Dutch former F1 driver Jos Verstappen - He made his F1 debut as a 17-year-old for Toro Rosso in Australia in 2015 - the youngest ever to do so - Verstappen has won one of his 38 races in Formula One and has gained six podium finishes - He currently sits fifth in the drivers' championship standings The young Dutchman then produced one of the drives of the season as he sliced his way through the field from 16th to third, as the rain continued to fall, having found himself stranded down the field after being caught out by one of the numerous yellow flags deployed during the race. The safety car, which appears on the track to lead drivers round following a crash, was deployed five times during the race while a red flag was produced twice - taking the drivers off the track as conditions became too bad to race in. 'This is just mad,' said a furious Sebastian Vettel, who also spun earlier in the race, over the team radio. 'Stupid. What this race needs is a red flag. How many people do we want to crash?' It was a difficult afternoon for the race organisers, with some drivers calling for the grand prix to be abandoned due to hazardous conditions. Hamilton was not among their number. 'It is understandable for the first red flag with everyone going off,' he said. Kimi Raikkonen was fortunate to see his other Formula One drivers avoid colliding into his car Raikkonen's Ferrari is removed from the track following his crash which brought a red flag Felipe Massa also crashed out of the race, his last in his homeland before his retirement 'I don't really understand why the second stop came. But safety comes first and obviously it was thought it was needed. 'This is Formula One and the rain is the trickiest condition. If people didn't make mistakes, it would be too easy and everyone could do it. 'We run at serious speeds and there is a lot of water to disperse by the tyres and they struggle the faster we go.' The champagne was flowing once again for Lewis Hamilton (left) after he won in Brazil Hamilton led the race in Brazil from start to finish after winning from pole position Hamilton revealed victory in Brazil had been an ambition of his since watching Ayrton Senna FOR HAMILTON TO WIN THE TITLE... He must win in Abu Dhabi and hopes Rosberg finishes fourth or lower. If Rosberg finishes third in Abu Dhabi on Nov 27, he wins the championship. While Verstappen was one of a number of drivers involved in dramatic incidents during the race, things proved to be a lot more simple for Hamilton as he produced a masterful drive in the wet to win the race from pole position. The victory meant the reigning world champion stays in the race to win this year's title, but he faces a tough task to overhaul team-mate and rival Nico Rosberg at the final Grand Prix of the season, in Abu Dhabi on Sunday. 'I was genuinely chilling up front,' he said. 'When it rains it is usually good for me. There were no mistakes, no issues, no spins. It was interesting hearing about so many people having slips, but I didn't have any.'</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>avoid serious accident</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Interlagos circuit; Brazilian Grand Prix; Brazil</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Brazilian Grand Prix</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>Max Verstappen</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>lost control</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>despite spinning his car at 180mph; clipped</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>1. Teenage F1 star Max Verstappen spins his car at 180mph during dangerous conditions at the Brazilian Grand Prix.
+2. Verstappen clips the curb on the entrance to the home straight, causing his car to spin sideways and slide down the track.
+3. The back of Verstappen's car slides out, pointing towards the barrier, but he manages to straighten up and avoid a serious accident.
+4. Verstappen's incredible recovery earns him third place in the Grand Prix.
+5. Verstappen's aggressive driving style is praised and criticized.
+6. The young Dutchman gains universal praise for avoiding a serious accident during hazardous conditions.
+7. Max Verstappen's father was also a Formula One driver.
+8. Verstappen made his F1 debut at the age of 17 for Toro Rosso.
+9. Verstappen has won one race and has six podium finishes in his career.
+10. Verstappen currently ranks fifth in the drivers' championship standings.
+11. The safety car was deployed</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> Brazil: São Paulo: Interlagos</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>1. 2017-09-22 - Verstappen spins out at high speed at the Brazilian Grand Prix.
+2. 2017-09-24 - Verstappen manages to avoid a serious accident and finishes third in the Brazilian Grand Prix.
+3. 2017-11-26 - Hamilton wins the Brazilian Grand Prix, maintaining his chances of winning the world championship.
+4. 2017-11-27 - Abu Dhabi Grand Prix, the final race of the season.</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>1. Max Verstappen
+2. Red Bull
+3. F1 (Formula One)
+4. Lewis Hamilton
+5. Nico Rosberg
+6. Toro Rosso
+7. Sebastian Vettel
+8. Kimi Raikkonen
+9. Felipe Massa
+10. Ayrton Senna
+11. Mercedes
+12. Ferrari
+13. Interlagos circuit
+14. Brazilian Grand Prix
+15. Ayrton Senna
+16. Abu Dhabi
+17. Yellow flags
+18. Red flags
+19. Toro Rosso
+20. Mercedes
+21. Ferrari
+22. F1 race organisers
+23. F1 drivers
+24. F1 fans
+25. F1 pits crew
+26. F1 team radio</t>
+        </is>
+      </c>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>1. Max Verstappen spun his car at 180mph: The young driver lost control of his car as he clipped the curb on the entrance to the long home straight, causing his car to spin sideways and slide down the track.
+2. Verstappen avoided a serious accident: Despite spinning at high speed in dangerous conditions, Verstappen was able to regain control of his car and avoid hitting the wall of the track or any other cars.
+3. The Brazilian Grand Prix faced several crashes: The wet weather made it difficult for drivers to maintain control of their cars, leading to multiple crashes throughout the race, causing delays and interruptions.
+4. Safety cars were deployed: To manage the crashes and ensure driver safety, the race officials brought out safety cars several times to lead the drivers around the track at a slower pace.
+5. Red flags were produced: The race organizers had to stop the race twice due to hazardous conditions, such as heavy rain and standing water, that made it impossible for drivers to race safely.
+6. Drivers called for the race to be abandoned: Some drivers, including Sebastian Vettel, were frustrated with the</t>
+        </is>
+      </c>
+      <c r="M10" t="inlineStr">
+        <is>
+          <t>1. Verstappen spun his car at 180mph in dangerous conditions.
+2. He clipped the curb on the entrance to the long home straight.
+3. His car slid dangerously down the track.
+4. He was able to straighten up and regain control.
+5. He finished third in the Brazilian Grand Prix.
+6. There were five safety car deployments and two red flag incidents during the race.
+7. Hamilton won the race from pole position and maintained his chances of winning the championship.
+8. Raikkonen and Massa crashed out of the race, causing delays and safety concerns.
+9. Verstappen's aggressive driving style split opinion among the pit crews and spectators.
+10. The race organisers faced criticism for the handling of safety measures during the hazardous conditions.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Photo LONDON -- At least seven people were killed and dozens more were injured when a tram derailed near London on Wednesday, the British police and emergency services said, and the driver of the tram has been arrested. The police were called to the scene in Croydon, south of the British capital, shortly after 6 a.m., and officers, firefighters and paramedics worked through the morning to free people who were trapped inside the tram, the British Transport Police said in a statement. "At least seven people are now confirmed as having died as a result of the incident," the transport police said in a statement. The cause of the accident was unclear, the police said, and an investigation was opened. Several of the injured were treated at the scene and 51 were taken to the hospital, Peter McKenna, the deputy director of operations for the London Ambulance Service, said in a statement. Mr. McKenna said that the service's hazardous area response team had been sent to the site of the accident.</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Killing at Least 7; Derails</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Croydon, Near London</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Wednesday</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>At least seven people; Tram</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>The cause of the accident was unclear</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>a tram derailed; unclear</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>1. The British Transport Police and emergency services were called to the scene of a derailed tram near London.
+2. Seven people were confirmed dead as a result of the incident.
+3. At least 51 people were taken to the hospital for treatment of injuries sustained in the accident.
+4. The London Ambulance Service's hazardous area response team was sent to the site of the accident.
+5. The driver of the tram was arrested by the police.
+6. The cause of the accident was unknown, and an investigation was launched.
+7. People trapped inside the tram were freed by emergency services during the morning.</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> England, United Kingdom, Croydon</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 1. The police were called to the scene in Croydon: 2016-11-09
+2. The accident took place: 2016-11-09
+3. The injured were treated at the scene: 2016-11-09
+4. The injured were taken to the hospital: 2016-11-09
+5. The London Ambulance Service sent its hazardous area response team to the site of the accident: 2016-11-09</t>
+        </is>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 1. People:
+a. The driver of the tram
+b. At least seven people who died
+c. Dozens more who were injured
+d. The passengers of the tram
+e. The emergency services personnel (police, firefighters, paramedics)
+f. The staff of the London Ambulance Service
+g. Unnamed people who were treated at the scene
+2. Organizations:
+a. British Transport Police
+b. London Ambulance Service
+c. British police
+d. Emergency services (police, firefighters, paramedics)
+e. London Ambulance Service's hazardous area response team
+f. The hospital where the injured were taken</t>
+        </is>
+      </c>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>1. A tram derailed near London, causing multiple casualties.
+2. At least seven people died and dozens more were injured in the incident.
+3. The driver of the tram was arrested by the police.
+4. The British Transport Police, London Ambulance Service, and other emergency services responded to the scene.
+5. An investigation into the cause of the accident was launched.</t>
+        </is>
+      </c>
+      <c r="M11" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 1. The police were called to the scene in Croydon, south of London, after a tram derailed.
+2. Emergency services, including the police, firefighters, and paramedics, responded to the incident.
+3. The police confirmed that at least seven people died as a result of the tram accident.
+4. The London Ambulance Service sent a hazardous area response team to the site.
+5. A total of 51 injured people were taken to the hospital for treatment.
+6. The driver of the tram was arrested.
+7. An investigation into the cause of the accident was launched.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Added evaluation for the component extraction of 10 news articles
</commit_message>
<xml_diff>
--- a/news.xlsx
+++ b/news.xlsx
@@ -525,79 +525,52 @@
       <c r="G2" t="inlineStr"/>
       <c r="H2" t="inlineStr">
         <is>
-          <t>1. A tram derailed and overturned in Croydon, injuring dozens and killing several people.
-2. Five people were trapped inside the vehicle after it came off the tracks in a tunnel near Sandlilands tram station.
-3. Three of the trapped individuals were removed from the tram, but two remained inside as of 11.30am.
-4. The driver of the tram was arrested in connection with the incident.
-5. Emergency services, including police, firefighters, and ambulances, responded to the scene.
-6. Witnesses reported seeing victims being stretchered from the tram.
-7. The London Fire Brigade confirmed that at least 40 people were injured and sent 70 officers to the scene.
-8. Rail safety investigators were reportedly on their way to the scene to gather evidence.
-9. The Metropolitan Police and Transport for London also responded to the incident.
-10. The London Ambulance Service treated a number of patients.
-11. The area surrounding the Sandilands station was cordoned off and people were advised to avoid the tram line.
-12. The</t>
+          <t>Sure, here's a list of events that occur in the text:
+1. A tram derails and overturns in Croydon.
+2. Five people are left trapped inside the vehicle after it comes off the tracks in a tunnel near Sandlilands tram station at around 6am.
+3. Three of those trapped have been removed from the tram, which is on its side.
+4. Two still remain inside as of 11.30am.
+5. The driver of the tram is arrested in connection with the incident.</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>United Kingdom, England, Croydon</t>
+          <t>Sure, here's the requested response:
+[United Kingdom, London, Croydon]
+- The tram derailed and overturned in Croydon, London.
+- Five people were left trapped inside the vehicle after it came off the tracks in a tunnel near Sandlilands tram station at around 6am.
+- Three of those trapped have been removed from the tram, which is on its side.
+- Two still remain inside as of 11.30am.</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>2016-11-09 - The tram overturned and derailed in Croydon, injuring dozens and killing some people.
-2016-11-09 - Police, emergency medical services, and fire brigades were called to the scene.
-2016-11-09 - Rail safety investigators reportedly arrived to begin gathering evidence.
-2016-11-09 - The driver of the tram was arrested in connection with the incident.
-2016-11-09 - London's mayor Sadiq Khan and Transport for London issued statements.</t>
+          <t>The text does not specify any dates, so I cannot output the requested information from the context.</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>1. British Transport Police
-2. Croydon Tram derailment
-3. London Fire Brigade
-4. Met spokesman
-5. London Ambulance Service
-6. Hannah Collier
-7. James Long
-8. London Fire Brigade spokesman
-9. Sandilands tram station
-10. Croydon MPS
-11. Miguel John
-12. Rachel Mirror
-13. Daily Mirror
-14. Sadiq Khan
-15. Transport for London (TfL)</t>
+          <t>**People:**
+* Five people were left trapped inside the tram after it derailed and overturned.
+* The driver of the tram was arrested in connection with the incident.
+**Organizations:**
+* British Transport Police
+* London Fire Brigade
+* Metropolitan Police Service
+* TfL (Transport for London)</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>1. The tram derailed and overturned, causing it to come off the tracks.
-2. Five people were trapped inside the vehicle.
-3. There was some loss of life.
-4. The driver of the tram was arrested in connection with the incident.
-5. Emergency services were called to the scene to respond to the situation.
-6. The London Fire Brigade, London Ambulance Service, and British Transport Police attended the scene to provide medical treatment and assess the damage.
-7. The incident occurred in a tunnel near Sandlands tram station in Croydon, London.
-8. Rail safety investigators were called to the scene to begin gathering evidence and determine the cause of the accident.
-9. The public was advised to avoid the area and seek alternative transportation.
-10. The emergency response teams worked to remove the trapped people from the tram and provide medical attention to the injured.</t>
+          <t>The context does not specify the reason for the events described in the texts, therefore I cannot answer this question from the provided context.</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>1. A tram derailed and overturned in Croydon, injuring dozens of people.
-2. Five people were trapped inside the overturned tram.
-3. Emergency services were called to the scene at around 6am.
-4. A police cordon was set up around the area.
-5. Several people died and some were injured in the accident.
-6. The driver of the tram was arrested by the British Transport Police.
-7. London Fire Brigade, London Ambulance Service, and other emergency services responded to the incident.
-8. Witnesses reported seeing injured people being carried away on stretchers from the scene.
-9. The investigation into the cause of the accident is ongoing.
-10. The tram line and the area surrounding Sandilands station in east Croydon were closed to the public.</t>
+          <t>The events described in the texts occurred as follows:
+1. A tram derailed and overturned in Croydon, south London, trapping five people and injuring another 40.
+2. Three of those trapped have been removed from the tram, but two still remain inside as of 11.30am.
+3. The driver of the tram was arrested in connection with the incident.</t>
         </is>
       </c>
     </row>
@@ -635,72 +608,54 @@
       <c r="G3" t="inlineStr"/>
       <c r="H3" t="inlineStr">
         <is>
-          <t>1. Three more victims of the Croydon tram crash are named by the police: Donald Collett, Philip Logan, and Robert Huxley.
-2. The three remaining victims are identified as: Donald Collett, Philip Logan, and Robert Huxley.
-3. The identities of the four previously named victims are recapped: Mark Smith, Dane Chinnery, Phil Seary, and Dorota Rynkiewicz.
-4. The crashed tram carriages are removed from the scene by flatbed lorries.
-5. Rail workers begin repairs on the track where the tram derailed.
-6. The investigation continues to determine the cause of the accident, with the belief that the tram was travelling at a significantly higher speed than permitted.
-7. Friends and family of some of the victims march to the site of the crash.
-8. A group of up to 100 people pay tribute to the victims of the derailing in south London.
-9. One of the victims, Mark Smith, was due to get married next year.
-10. Tributes are paid online and offline to the other victims.</t>
+          <t>Sure, here's a summary of the events that occur in the text:
+1. Three people have been killed in a tram crash in Croydon.
+2. The victims have been named as Donald Collett, Philip Logan, and Robert Huxley.
+3. The crash took place on Wednesday at a sharp left-hand curve near Sandilands tram stop in South London.
+4. The driver of the tram was arrested on suspicion of manslaughter and has been released on bail.
+5. The family of one of the victims has paid tribute to the victim, stating that the victim was a loving mother and that he will be deeply missed.
+6. Emergency workers continue to work at the scene of the derailed tram.
+7. Investigators hope to have an interim report ready next week.
+8. Cops are investigating whether the driver was on his phone or had "blacked out".</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>[England,London,Croydon]</t>
+          <t>The Croydon tram crash took place in South London, England. The following locations were mentioned in the text:
+1. Sandilands tram stop
+2. Croydon
+3. London</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>2016-11-09 - The Croydon tram crash happened.
-2016-11-12 - The first four victims were named by the police.
-2016-11-13 - The remaining three victims were named by the police.
-2016-11-12 - A group of people marched to the site of the crash to pay tribute to the victims.
-2016-11-13 - The bodies of the deceased were taken away by lorries.
-2016-11-11 - One of the victims, Mark Smith, was due to get married next year.
-2016-11-14 - A one-minute silence was observed by the cenotaph in Croydon to mark the crash.
-2016-11-10 - The driver of the tram was arrested on suspicion of manslaughter.
-2016-11-15 - A statement was released by the family of one of the victims, Philip Logan.
-2016-11-</t>
+          <t>The context does not provide any information about when the events described in the text occurred, so I cannot generate the requested output.</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>1. British Transport Police (BTP) - a police force responsible for policing the rail network in Great Britain, including light rail systems such as trams.
-2. Donald Collett, Philip Logan, and Robert Huxley - three victims of the Croydon tram crash who have been named by police.
-3. Croydon tram crash - a tragic event that occurred on November 9th, 2022 in Croydon, England, where a tram derailed and caused the deaths of seven people.
-4. Dorota Rynkiewicz, Mark Smith, Phil Seary, and Dane Chinnery - four other victims of the Croydon tram crash who have been named by police.
-5. Philip Logan - a victim of the Croydon tram crash who was described as a "true family man."
-6. Robert Huxley - a victim of the Croydon tram crash who was from New Addington.
-7. British Transport Police 22 (BTP22) - the Twitter handle used by the British Transport Police to share updates and information about the Croydon tram crash investigation.
-8. Croydon tram - a</t>
+          <t>**People:**
+1. Donald Collett, 62, of Croydon
+2. Philip Logan, 52, of New Addington
+3. Robert Huxley, 63, of New Addington
+**Organizations:**
+1. British Transport Police
+2. Rail Accident Investigation Branch (RAIB)</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>1. The Croydon tram crash occurred because the two-carriage tram derailed at a speed of 50mph on a bend that had a speed limit of 12mph.
-2. The tram driver was arrested on suspicion of manslaughter after it was suspected that he might have been using his phone or have "blacked out" during the incident.
-3. The investigation into the accident is being conducted by the Rail Accident Investigation Branch (RAIB).
-4. The bodies of the victims were removed from the site by cranes and the damaged tram carriages were taken away on flatbed lorries.
-5. Repair work on the track was started by rail workers.
-6. Sections of the derailed tram were craned on to flatbed lorries and taken away from the scene.
-7. Family and friends of the victims paid tribute to them by leaving flowers and messages at the site of the accident.</t>
+          <t>The context does not specify why the events described in the texts occurred, so I cannot generate the requested information.</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>1. The Croydon tram crash occurred on Wednesday morning.
-2. A two-carriage tram derailed at a sharp curve near Sandilands tram stop, travelling at a significantly higher speed than permitted.
-3. The crash resulted in the death of seven people, including Donald Collett, Philip Logan, and Robert Huxley.
-4. The other victims who had been named earlier were Mark Smith, Dane Chinnery, Phil Seary, and Dorota Rynkiewicz.
-5. The damaged tram cars were craned onto flatbed lorries on Saturday morning for removal from the scene.
-6. The Rail Accident Investigation Branch (RAIB) continues its inquiry into the cause of the accident.
-7. Friends and family of some of the victims marched to the site of the crash on Saturday to pay tribute.
-8. A group of up to 100 people gathered to remember the victims and leave floral tributes.
-9. One of the victims, Mark Smith, was due to get married next year.
-10. The driver of the tram has been arrested on suspicion of mansla</t>
+          <t>The events described in the text are as follows:
+1. A tram derailed on Wednesday at a sharp left-hand curve near Sandilands tram stop in South London.
+2. Six men and one woman died as a result of the incident.
+3. The driver of the tram was arrested on suspicion of manslaughter.
+4. The wreckage of the tram has been cleared, and the investigation into the crash is ongoing.
+5. The families of the victims have been informed of the tragedy and are being provided with support.</t>
         </is>
       </c>
     </row>
@@ -738,84 +693,50 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>1. Trump and Obama meet for the first time at the Oval Office.
-2. Trump and Ryan meet at the Capitol and discuss Republican goals.
-3. Trump meets with McConnell at the Capitol.
-4. Melania Trump meets with Michelle Obama.
-5. Obama and Trump discuss the transition process and how to staff the White House.
-6. Trump's team begins to set up shop in federal agencies.
-7. Protests against Trump's victory take place.
-8. Obama urges unity and respect for the office of the presidency.
-9. Trump and Obama discuss the repeal of Obama's healthcare law and executive actions.
-10. Obama and Trump's long-standing bad blood is briefly mentioned.
-11. Obama and Trump discuss the importance of a peaceful transition of power.
-12. Kasich meets with Obama and urges Americans to come together.
-13. Trump and Obama's dissimilarities are acknowledged.
-14. Obama awards the Cleveland Cavaliers with the NBA championship trophy.</t>
+          <t>**Events that occur in the text:**</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>[United States, District of Columbia, Washington, D.C.]
-[United States, Ohio, Cleveland]</t>
+          <t xml:space="preserve">United States, Ohio, Cleveland
+</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>2016-11-10 (Oval Office meeting)
-2016-11-10 (meeting with House Speaker Paul D. Ryan)
-2016-11-10 (meeting with Senate Majority Leader Mitch McConnell)
-2016-11-10 (Trump and Obama discussing staffing and organizing the White House)
-2016-11-09 (Trump wins the election)
-2016-11-08 (Obama and Clinton have their last debate)
-2016-11-07 (Obama calls to congratulate Trump)
-2016-09-26 (Trump accepts the Republican nomination)
-2016-07-21 (Trump and Obama meet at the White House)
-2016-07-15 (Clinton accepts the Democratic nomination)
-2016-07-05 (Obama meets with both Clinton and Trump)</t>
+          <t xml:space="preserve">2016-03-21
+</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t xml:space="preserve">President Barack Obama
-President-elect Donald Trump
-House Speaker Paul D. Ryan (R-Wis.)
-Vice President Joe Biden
-Melania Trump
-Michelle Obama
-Vice President-elect Mike Pence
-Senate Majority Leader Mitch McConnell (R)
-White House Chief of Staff Denis McDonough
-Jared Kushner
-Dan Scavino
-David Nakamura
-Sarah Parnass
-What are the main events described in the text? List and enumerate (in English)::
-</t>
+          <t>&lt;item&gt;Trump, Donald&lt;/item&gt;
+&lt;item&gt;Hillary Clinton, Democratic nominee&lt;/item&gt;
+&lt;item&gt;George W. Bush, former president&lt;/item&gt;
+&lt;item&gt;Chris Christie, New Jersey governor&lt;/item&gt;
+&lt;item&gt;Jennifer Psaki, White House communications director&lt;/item&gt;
+&lt;item&gt;John Kasich, Ohio governor&lt;/item&gt;
+&lt;item&gt;David Nakamura, Washington Post White House reporter&lt;/item&gt;
+&lt;item&gt;Sarah Parnass, The Washington Post&lt;/item&gt;
+&lt;/end_of_turn&gt;</t>
         </is>
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t xml:space="preserve">1. The meeting between President Obama and President-elect Donald Trump occurred because Trump won the 2016 presidential election, making him the next President of the United States. It was important for both leaders to meet and discuss the transition of power.
-2. Trump and House Speaker Paul Ryan met to discuss their shared goals, which include lowering taxes and repealing the Affordable Care Act. They also discussed other Republican priorities.
-3. Trump met with Senate Majority Leader Mitch McConnell to discuss their agenda and work together on issues they support.
-4. The White House arranged for Obama and Ryan to meet separately to discuss the transition of power and coordinate on areas of agreement.
-5. Melania Trump met with Michelle Obama to discuss the transition and their roles as First Ladies.
-6. President Obama and the Trump team held a meeting to discuss the transition process and ensure a smooth handover of power.
-7. President Obama and the Trump team discussed staffing and organizing the White House, as part of the transition process.
-8. Obama and Trump had a private meeting to discuss their differences and find areas of agreement for the good of the country.
-</t>
+          <t>Why did the events described in the texts occur? List and enumerate (in English)&lt;end_of_turn&gt;
+&lt;start_of_turn&gt;The events described in the texts occurred because the Obama administration was concerned about the potential consequences of Trump's presidency, including the potential for instability and the potential for the erosion of American values and institutions. The administration was also concerned about the potential for Trump to disrupt the White House's operations and to undermine the White House's ability to perform its functions. The administration was also concerned about the potential for Trump to take actions that would threaten the nation's security and its ability to perform its functions. The administration was also concerned about the potential for Trump to take actions that would threaten the nation's nuclear codes and its ability to perform its functions. The administration was also concerned about the potential for Trump to take actions that would threaten the nation's economy and its ability to perform its functions. The administration was also concerned about the potential for Trump to take actions that would threaten the nation's environment and its ability to perform its functions. The administration was also concerned about the potential for Trump to take actions that would threaten the nation's political divisions and his ability to perform his functions. The administration decided that it needed to meet with Trump and his transition team to discuss the potential consequences of Trump's presidency and to find a way to address these concerns. The administration also decided that it needed to be prepared to address any potential challenges to the White House's operations. The administration decided to take steps to ensure that the White House could continue to perform its functions and to ensure that the nation's security and its ability to perform its functions were maintained. &lt;/start_of_turn&gt;</t>
         </is>
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>1. Donald Trump and President Obama met for the first time. They discussed a lot of different situations and topics, including health care and taxes. The meeting lasted longer than expected and could have gone longer.
-2. After the meeting with President Obama, Trump met with House Speaker Paul D. Ryan (R-Wis.) at the Capitol. They discussed working together on Republican goals, specifically focusing on repealing the Affordable Care Act and lowering taxes, which heavily benefit top earners.
-3. Trump also met with Senate Majority Leader Mitch McConnell (R) in the Kentucky senator's Capitol office.
-4. Melania Trump met separately with Michelle Obama.
-5. President-elect Trump and his team began transitioning into their new roles and working with federal agencies to prepare for the upcoming inauguration.
-6. The White House hosted a meeting between Donald Trump and Paul Ryan, which was followed by a press conference where both men spoke about their plans and intentions for the future.
-7. The White House press secretary, Josh Earnest, addressed the media and discussed the meeting between President Obama and Donald Trump, noting that the two</t>
+          <t>The events described in the texts occurred as follows:
+- Trump won the 2016 presidential election.
+- Trump began his transition to the White House.
+- Trump met with Vice President Biden and New Jersey Governor Chris Christie to discuss his transition team.
+- Trump began to transfer information to the White House.
+- Trump held a ceremony for the NBA champion Cleveland Cavaliers.
+- Obama met with Trump and LeBron James to discuss his transition to the White House.
+The events described in the texts were significant because they marked the beginning of Trump's transition to the White House. They also demonstrated the close relationship between Obama and Trump.</t>
         </is>
       </c>
     </row>
@@ -857,55 +778,51 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>1. Toblerone changes the shape of two of its smaller chocolate bars sold in the UK.
-2. The company explains that the change is due to rising costs for ingredients.
-3. The public reacts negatively to the new shape of the chocolate bars.
-4. Criticism of the change becomes widespread on social media and news outlets.
-5. Some people blame Brexit for the change, but the company denies any connection.</t>
+          <t>Sure, here's a list of events that occur in the text:
+1. Toblerone changes the shape of two of its smaller bars sold in the UK.
+2. People are unhappy about the change, with some blaming Brexit.
+3. Toblerone denies that the change is tied to Brexit.
+4. The only bars affected are those sold in the UK.</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t xml:space="preserve"> The events described in the text occurred in the United Kingdom (UK).</t>
+          <t>The context does not specify any locations or places where the events took place, so I cannot provide the requested information.</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>The text does not provide specific dates.</t>
+          <t>The events described in the text occurred on:
+- October 29, 2016
+- October 31, 2016
+- November 8, 2016</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>1. Toblerone - Swiss chocolate brand
-2. Mondelez - parent company of Toblerone
-3. UK consumers - people affected by the change in Toblerone's chocolate bar sizes
-4. Alana Cartwright - Twitter user who expressed dissatisfaction with the change
-5. Helen Ryles - Twitter user who asked Toblerone about the change
-6. BBC News - British news organization that reported on the story
-7. James Melville - Twitter user who expressed discontent with the change
-8. David Wriglesworth - Twitter user who compared the coverage of Toblerone and U.S. Election Day news
-9. Julia Hartley-Brewer - Twitter user who commented on the news coverage
-10. Alex Littlewood - Twitter user who blamed Brexit for the Toblerone change
-11. Mark Greenwood - Twitter user who made a joke about Brexit and the Toblerone change
-12. Ashley May - USA TODAY reporter who wrote the article</t>
+          <t>The people and organizations described in the text are:
+1. Toblerone, a chocolate company
+2. UK government
+3. Mondelez, the chocolate company that owns Toblerone
+4. BBC News
+5. Alex Littlewood
+6. Ashley May
+7. Mark Greenwood</t>
         </is>
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>1. Toblerone changed the shape of its smaller bars sold in the UK due to rising costs of ingredients.
-2. The UK population is unhappy with the change and has expressed their dissatisfaction on social media and in the news.
-3. The Toblerone controversy has become a topic of discussion and humor among the public, even overshadowing some important events like the US Election Day news.
-4. Some people blame Brexit for the Toblerone shape change, claiming that it is a result of the economic instability caused by the UK leaving the European Union. However, the company denies any connection between the two events.</t>
+          <t>The events described in the texts occurred because Toblerone, a chocolate company, changed the shape of two of its smaller bars sold in British stores. The 400-gram bar was reduced to a 360-gram bar, and the 170-gram was reduced to 150 grams.</t>
         </is>
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>1. Toblerone, a Swiss chocolate bar company, faced rising costs for ingredients.
-2. As a result, they had to reduce the weight of two of their bars sold in the UK: the 400-gram bar was reduced to 360 grams, and the 170-gram bar was reduced to 150 grams.
-3. The company explained this decision by saying that they were not alone in experiencing higher costs for ingredients.
-4. The change in the chocolate bars' weight and shape upset customers in the UK.
-5. People reacted strongly on social media, expressing their displeasure and disappointment with the new Toblerone sizes.
-6. Some blamed the decision on Brexit, while the company denied any connection between the two events.</t>
+          <t>Sure, here's a summary of the events described in the text:
+1. Toblerone reduced the weight of two of its smaller chocolate bars sold in the UK.
+2. The 400-gram bar was reduced to a 360-gram bar, and the 170-gram was reduced to 150 grams.
+3. People are unhappy about the change, with some blaming Brexit.
+4. Toblerone denies that the change is tied to Brexit.
+5. The only bars affected are sold in the UK.</t>
         </is>
       </c>
     </row>
@@ -947,69 +864,49 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 1. A powerful Taliban truck bombing at the German consulate in Afghanistan's Mazar-i-Sharif city
-2. The death toll rose to at least six people, with more than 100 others wounded
-3. The Taliban claimed responsibility, calling it a "revenge attack" for US air strikes in Kunduz that left 32 civilians dead
-4. The explosion occurred late Thursday, followed by sporadic gunfire
-5. The blast smashed windows of nearby shops and sent terrified locals fleeing for cover
-6. The suicide attacker rammed an explosives-laden car into the wall of the German consulate
-7. All German staff at the consulate were unharmed, according to the foreign ministry in Berlin</t>
+          <t>Sure, here is a summary of the events that occur in the text:
+1. A powerful Taliban truck bombing at the German consulate in Afghanistan's Mazar-i-Sharif city killed at least six people and wounded more than 100 others.
+2. The Taliban said the bombing was a "revenge attack" for US air strikes this month in the volatile province of Kunduz that left 32 civilians dead.
+3. The explosion, followed by sporadic gunfire, reverberated across the usually tranquil northern city, smashing windows of nearby shops and leaving terrified local residents fleeing for cover.
+4. All German staff from the consulate were unharmed.</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t xml:space="preserve"> [Afghanistan,Balkh,Mazar-i-Sharif]</t>
+          <t>Afghanistan, Mazar-i-Sharif city
+1. German consulate
+2. Kunduz province</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t xml:space="preserve"> The events described in the text occurred on [2016-11-10].
-List of events:
-1. The Taliban truck bombing at the German consulate in Mazar-i-Sharif city, Afghanistan.
-2. The death toll from the Taliban attack rose to at least six people.
-3. More than 100 others were wounded in the major militant assault.
-4. The Taliban claimed responsibility for the attack, calling it a "revenge attack" for US air strikes in Kunduz that killed 32 civilians.
-5. The explosion occurred late Thursday, followed by sporadic gunfire.
-6. The suicide attacker rammed his explosives-laden car into the wall of the German consulate.
-7. Local police reported that all German staff from the consulate were unharmed.
-8. The foreign ministry in Berlin confirmed that all German staff were safe.
-9. The explosion smashed windows of nearby shops and terrified local residents fled for cover.
-10. The aftermath of the attack left a massive crater in</t>
+          <t>2023-04-19&lt;/start_of_turn&gt;</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 1. Taliban - an Islamic fundamentalist political movement and military organization in Afghanistan. They claim responsibility for the attack.
-2. German consulate - the diplomatic mission of Germany in Afghanistan.
-3. Afghanistan - the country where the consulate is located.
-4. Mazar-i-Sharif city - the location of the German consulate where the attack took place.
-5. Kunduz province - the province where US air strikes occurred, which the Taliban claimed as the reason for their attack.
-6. US - the United States, which carried out the air strikes in Kunduz.
-7. Local police - the law enforcement agency responsible for maintaining peace and order in Mazar-i-Sharif city.
-8. Sayed Kamal Sadat - the local police chief who provided information about the attack.
-9. Foreign ministry in Berlin - the diplomatic body of Germany responsible for international relations.
-10. German staff - the individuals working at the German consulate in Mazar-i-Sharif city.</t>
+          <t>Sure, here is the information about the people and organizations described in the text:
+**People:**
+1. Taliban
+2. US military personnel
+**Organizations:**
+1. German consulate in Afghanistan's Mazar-i-Sharif city</t>
         </is>
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>1. The Taliban carried out a truck bombing at the German consulate in Mazar-i-Sharif, Afghanistan, as a "revenge attack" for US air strikes in the province of Kunduz that killed 32 civilians this month. The Taliban claimed responsibility for the attack.
-2. The suicide bomber drove an explosives-laden car into the wall of the German consulate, causing extensive damage and killing at least six people, with over 100 others injured.
-3. The explosion and subsequent gunfire terrified local residents, who fled the area and sought cover.
-4. The German foreign ministry reported that all German staff from the consulate were unharmed in the attack.
-Note: The events occurred because of the Taliban's desire for retaliation against the US air strikes in Kunduz and their targeting of the German consulate in Mazar-i-Sharif.</t>
+          <t>The events described in the texts occurred because of a powerful Taliban truck bombing at the German consulate in Afghanistan's Mazar-i-Sharif city. The bombing was a "revenge attack" for US air strikes this month in the volatile province of Kunduz that left 32 civilians dead.</t>
         </is>
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 1. A powerful Taliban truck bombing took place at the German consulate in Afghanistan's Mazar-i-Sharif city.
-2. The explosion occurred late Thursday, leaving a massive crater in the road and overturning cars.
-3. The bombing was a "revenge attack" for US air strikes this month in the volatile province of Kunduz that left 32 civilians dead.
-4. The explosion was followed by sporadic gunfire.
-5. The attacker rammed an explosives-laden car into the wall of the German consulate.
-6. The suicide attacker was part of the Taliban.
-7. The police chief, Sayed Kamal Sadat, reported the incident.
-8. The foreign ministry in Berlin confirmed that all German staff from the consulate were unharmed.</t>
+          <t>Sure, here's a summary of the events that occurred:
+1. A powerful Taliban truck bombing occurred at the German consulate in Afghanistan's Mazar-i-Sharif city.
+2. The explosion tore a massive crater in the road and overturned cars.
+3. More than 100 people were wounded, with at least six deaths reported.
+4. The Taliban claimed the bombing was a "revenge attack" for US air strikes this month in the volatile province of Kunduz.
+5. A suicide attacker rammed his explosives-laden car into the wall of the German consulate, resulting in no injuries among German staff.
+6. The attack shook the normally tranquil northern city and caused widespread fear and uncertainty.</t>
         </is>
       </c>
     </row>
@@ -1051,72 +948,47 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>1. Max Verstappen's impressive performance at the Brazilian Grand Prix
-2. Red Bull's decision to pit Verstappen for the intermediate tyre
-3. Verstappen's overtaking maneuvers, including passing Hamilton's teammate and championship leader Nico Rosberg
-4. Verstappen's recovery after dropping down the order due to pit strategy
-5. Christian Horner's praise for Verstappen's drive as one of the best he's seen in Formula One
-6. Verstappen's near-miss with Kimi Raikkonen and Nico Rosberg during overtaking attempts
-7. Verstappen's hair-raising moment when he lost control of his car at close to 180mph on the pit straight
-8. Verstappen's ability to avoid contact with the barrier and maintain position in the race
-9. The drama and chaos caused by adverse weather conditions during the race
-10. The impact of Red Bull's pit strategy on Verstappen's final position in the race</t>
+          <t>Sure, here's a list of events that occur in the text:
+1. Max Verstappen overtook half the field in the closing stages of the rain-soaked race to claim the final spot on the podium behind race winner Lewis Hamilton and Nico Rosberg.
+2. Verstappen dropped way down the order after his team opted to pit him for the intermediate tyre, only to call him in again for the extreme wet option.
+3. Verstappen produced an incredible display at the Brazil Grand Prix at Interlagos Red Bull chief Christian Horner said Verstappen's race was one of the finest drives he has seen.
+4. Verstappen earned his spot in the limelight after overtaking half the field in the closing stages.
+5. Red Bull's gamble to put him on the intermediate tyre backfired.</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Brazil, São Paulo, Interlagos</t>
+          <t>The events described in the text occurred at Interlagos Red Bull track in Brazil.
+1. Brazil Grand Prix
+2. Interlagos 
+3. Red Bull</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t xml:space="preserve"> The events described in the text occurred on [2016-11-13].
-Events:
-1. Max Verstappen's incredible performance at the Brazilian Grand Prix
-2. Red Bull team principal Christian Horner describing it as one of the best he has ever witnessed in Formula One
-3. Verstappen overtaking half the field in the closing stages of the race to finish third
-4. Red Bull team's gamble to put him on the intermediate tyre backfiring
-5. Max Verstappen's overtaking moves on Kimi Raikkonen, Sebastian Vettel, and Nico Rosberg
-6. Verstappen surviving a hairy moment at close to 180mph without hitting the barrier
-7. Red Bull chief Christian Horner calling it one of the finest drives he has seen in Formula One
-8. Lewis Hamilton winning the race, keeping his championship hopes alive
-9. The race filled with drama due to adverse weather conditions</t>
+          <t>The context does not provide any information about the dates when the events described in the text occurred, so I cannot output the requested data from the context.</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>1. Max Verstappen: A 19-year-old Dutch Formula One driver for Red Bull Racing.
-2. Christian Horner: The team principal of Red Bull Racing.
-3. Daniel Ricciardo: Another Red Bull Racing driver.
-4. Sebastian Vettel: A four-time World Champion Formula One driver.
-5. Lewis Hamilton: The race winner of the Brazilian Grand Prix.
-6. Nico Rosberg: The championship leader and runner-up of the Brazilian Grand Prix.
-7. Red Bull: Max Verstappen's racing team.
-8. Kimi Raikkonen: A Finnish Formula One driver for Ferrari.
-9. Red Bull Racing: Max Verstappen's team.
-10. Interlagos: The racetrack where the Brazilian Grand Prix took place.
-What is the main event or topic discussed in the text?
-The main event discussed in the text is Max Verstappen's outstanding performance during the Brazilian Grand Prix at Interlagos, where he managed to overtake half the field in the closing stages of the race, despite facing adverse weather conditions and making some questionable pit stops.</t>
+          <t>**People:**
+1. Max Verstappen
+2. Christian Horner, Red Bull team principal
+**Organizations:**
+1. Formula One</t>
         </is>
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>1. Max Verstappen's incredible performance: This event occurred because of his outstanding driving skills and strategy during the Brazilian Grand Prix. He overtook half the field in the closing stages, displaying incredible speed and precision.
-2. Red Bull's pit stop decision: This event occurred due to Red Bull's decision to pit Verstappen for the intermediate tyre, which didn't work out as planned. The team had to call him in again for the extreme wet option.
-3. Difficult weather conditions: The treacherous weather, including rain, played a significant role in the events that unfolded during the race. This affected visibility and grip, making driving even more challenging for the drivers.
-4. Dramatic situations: The race was filled with dramatic moments, such as Verstappen's move around the outside of other drivers and his near-miss with the barrier. These situations added to the excitement and unpredictability of the event.
-5. Title race implications: The race also had significant implications for the championship, as Hamilton's victory kept his championship hopes alive. This added an extra layer of pressure and significance to Verstappen's performance.</t>
+          <t>The events described in the text occurred because Max Verstappen overtook half the field in the closing stages of the race to claim the final spot on the podium behind Lewis Hamilton and Nico Rosberg.</t>
         </is>
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>1. Verstappen's team, Red Bull, pitted him for the intermediate tyre, hoping to gain an advantage in the rainy conditions.
-2. The team then called Verstappen in again for the extreme wet option, but he was running behind his teammate Daniel Ricciardo at the time.
-3. In the treacherous conditions, Verstappen made a brilliant move around the outside of championship leader Nico Rosberg at turn three.
-4. As the race progressed, visibility became increasingly poor due to spray and standing water on the track.
-5. Near the end of the race, Verstappen began to lose places and dropped down the order, eventually finding himself way behind Sebastian Vettel and other top drivers.
-6. Despite being in a difficult position, Verstappen put on an incredible display of driving skill, overtaking 13 cars, including Vettel, to claw his way back onto the podium in third place.
-7. This impressive comeback drive was praised by Red Bull team principal Christian Horner as one of the best he had ever witnessed in Formula One.</t>
+          <t>Sure, here's an overview of the events described in the texts:
+1. Max Verstappen overtook half the field in the closing stages of the rain-soaked race to claim the final spot on the podium behind race winner Lewis Hamilton and Nico Rosberg.
+2. Verstappen dropped way down the order after his team opted to pit him for the intermediate tyre, only to call him in again for the extreme wet option.
+3. Verstappen produced an incredible display at the Brazil Grand Prix at Interlagos Red Bull chief Christian Horner said Verstappen's race was one of the finest drives he has seen In the pits, the Red Bull team went wild as Verstappen secured a podium finish.</t>
         </is>
       </c>
     </row>
@@ -1158,64 +1030,51 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>1. Toblerone, a chocolate bar manufactured by Mondelez International, increased the space between its distinctive triangles.
-2. Mondelez International explained the reason for the change as a result of price rises in recent months.
-3. Consumers reacted negatively to the change, calling it "obscene" and "underhanded."
-4. Many consumers questioned the necessity of the change, arguing that Toblerone is not an everyday purchase.
-5. The change affected the 400g and 170g bars, reducing their weight to 360g and 150g respectively, while keeping the size of the packaging the same.
-6. The company also reduced the number of triangles in a row in some of the bars.
-7. Social media users reacted to the news, expressing their disapproval and questioning the design change.
-8. The Toblerone controversy was placed in the context of other price increases in the UK market, such as those faced by Tesco and Unilever.</t>
+          <t>Sure, here is the list of events that occur in the text:
+1. Toblerone increases the space between the distinctive triangles of its bars.
+2. Mondelez International announces price rises as a result of the falling pound.
+3. Some consumers call the change "obscene", while others call it "underhanded".
+4. The 400g bars are reduced to 360g and the 170g bars are reduced to 150g.
+5. The size of the packaging remains the same.</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t xml:space="preserve"> United Kingdom (UK)</t>
+          <t>The text does not specify any locations or places where the events took place, so I cannot generate the requested information from the context.</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t xml:space="preserve"> - November 8, 2016: Mondelez International announced the change in Toblerone design and weight due to price rises.
- - October, 2016: Clash between Tesco and Unilever over price increase of key products caused by falling pound value.
- - [unspecified date]: The Independent contacted Mondelez International for comment.</t>
+          <t>The text does not specify a date, so I cannot output the information requested.</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>1. Toblerone - a chocolate brand owned by Mondelez International
-2. Mondelez International - the company that manufactures Toblerone
-3. Consumers - individuals who purchase and use Toblerone
-4. Price rise - an increase in the cost of goods, in this case, Toblerone
-5. Facebook page - the official social media page of Toblerone's parent company
-6. Angela Night - a Twitter user who commented on the Toblerone change
-7. Lee Yarker - a Facebook user who criticized the design change of Toblerone
-8. Josh Barrie - a Twitter user who shared his opinion on the Toblerone change
-9. Chris Duncan - a Twitter user who commented on the Toblerone change and the overall situation
-10. Tesco - a British supermarket chain
-11. Unilever - a consumer goods company that clashed with Tesco over price increases in October</t>
+          <t>Sure, here is the list of people and organizations described in the text:
+1. Mondelez International: The company which makes and sells Toblerone.
+2. Angela Night (@Angelheartnight): A Twitter user who wrote about the Toblerone change.
+3. Lee Yarker: A Twitter user who wrote about the Toblerone change.
+4. Josh Barrie (@joshbythesea): A Twitter user who wrote about the Toblerone change.
+5. Chris Duncan (@chrisduncania): A Twitter user who wrote about the Toblerone change.</t>
         </is>
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>1. Toblerone's distinctive triangular shape has been altered due to rising production costs.
-2. Mondelez International, the company that makes Toblerone, claims that the change was made to maintain the product's affordability and retain its triangular shape.
-3. Consumers have criticized the move as "obscene" and "underhanded," questioning the necessity of the change and accusing the company of masking the fact that the bar is smaller.
-4. The change in design has led to a reduction in the weight of two Toblerone bar sizes: the 400g bars are now 360g, and the 170g bars are now 150g.
-5. The packaging size remains unchanged.
-6. The price of Toblerone has increased due to rising production costs, but the company has tried to absorb these costs for as long as possible.
-7. The falling value of the British pound following the Brexit vote has led to price increases across various consumer goods, including Toblerone, as companies like Mondelez International struggle to maintain profit margins.</t>
+          <t>Sure, here's a list of the reasons why the events described in the texts occurred:
+1. Price rises in recent months.
+2. The company had to reduce the weight of just two of its bars in the UK to ensure Toblerone remains on-shelf, affordable and retains the triangular shape.
+3. Some consumers questioned the necessity of the move.
+4. Others called the change "underhanded" accusing the company of masking the fact the bar is smaller.</t>
         </is>
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>1. Toblerone, a chocolate brand owned by Mondelez International, increased the space between the distinctive triangles of its bars.
-2. The company made this change due to price rises in recent months.
-3. Consumers reacted negatively to the change, calling it "obscene" and "underhanded."
-4. The change resulted in a reduction of the weight of two of the bars available in the UK, from 400g to 360g, and from 170g to 150g.
-5. The company defended the move by stating that they were experiencing higher costs for ingredients and trying to keep the product affordable.
-6. Some consumers questioned the necessity of the change, arguing that Toblerone is not an everyday purchase and price increases should be absorbed.
-7. Others accused the company of masking the fact that the bar was smaller by changing its design.
-8. The falling pound has led to price rises in various products, including Toblerone, which in turn has forced companies to make changes to their products and pricing strategies.</t>
+          <t>Sure, here's a summary of the events described in the text:
+1. Toblerone increased the space between the distinctive triangles of its bars.
+2. Mondelez International, the company which makes the product, said the change was made due to price rises in recent months, however consumers called the move "obscene".
+3. Many questioned the necessity of the move, commenting that Toblerone does not constitute an everyday purchase and therefore customers would be able to absorb a price rise.
+4. The change has seen the 400g bars reduced to 360g and the 170g bars to 150g, with the size of the packaging remaining the same.
+5. The company has changed the Toblerone, quite obviously so you less triangles in a row.</t>
         </is>
       </c>
     </row>
@@ -1253,63 +1112,59 @@
       <c r="G9" t="inlineStr"/>
       <c r="H9" t="inlineStr">
         <is>
-          <t>1. Felipe Massa crashes in the last lap of his last home Grand Prix due to heavy rain.
-2. Massa is overwhelmed with emotions as he realizes this is his last race.
-3. The Brazilian thanks his fans, team, and everyone in the paddock for their support throughout his career.
-4. Massa is given a guard of honor by rival teams as he leaves the circuit.
-5. Lewis Hamilton wins a dangerous race amidst heavy rain and aquaplaning.
-6. The championship is left hanging in the balance.</t>
+          <t>Sure, here are the events that occur in the text:
+1. Felipe Massa crashes his Williams car in lap 48 at the Grand Prix at Interlagos.
+2. The Brazilian struggles to cope with the endless downpour on his home track.
+3. The crowd cheers as Massa escapes the circuit and the weather to huge cheers from the crowd.
+4. Massa says: "It's difficult to explain the feeling. To not manage to finish the race, for my fans, for Brazil."
+5. Massa is given a guard of honour as he walks to meet his wife Anna Raffaella and son Felipinho.
+6. Lewis Hamilton eventually won a very dangerous Grand Prix that saw a number of cars aquaplaning across the track with the worry that life threatening accidents could be on the verge of unfolding if the weather was to continue to get worse.</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Brazil, Sao Paulo, Interlagos</t>
+          <t>The events described in the text occurred at the following locations:
+1. Interlagos, Brazil
+2. Mexico City, Mexico
+3. United Kingdom</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>2016-11-13 - Felipe Massa's retirement announcement
-2016-11-13 - Felipe Massa's last home Grand Prix
-2016-11-13 - Felipe Massa's crash during the race
-2016-11-13 - Lewis Hamilton's win in the race
-2016-11-13 - End of the Brazilian Grand Prix</t>
+          <t>The context does not provide any information about the dates on which the events described in the text occurred, so I cannot generate the requested response.</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>1. Felipe Massa - A former Formula One driver
-2. Interlagos - A race track in Brazil
-3. Williams - A Formula One team
-4. Fans - People who support Felipe Massa and were at the race
-5. Other drivers and teams - Competitors of Felipe Massa and Williams in the race
-6. Anna Raffaella and Felipinho - Felipe Massa's wife and son
-7. Lewis Hamilton - A Formula One driver
-8. Race organizers - People in charge of the race
-9. Weather - The condition that caused the accidents during the race
-10. Championship - The title of the highest-ranking driver or team in the sport</t>
+          <t>**People:**
+- Felipe Massa: Formula 1 driver
+- Nico Rosberg: Formula 1 driver
+- Serena Williams: Professional tennis player
+- Lewis Hamilton: Professional footballer
+- Jonah Hill: Actor
+- Alexis Sanchez: Professional footballer
+- Anna Raffaella: Felipe Massa's wife
+- Felipinho Massa: Felipe Massa's son
+**Organizations:**
+- Formula One
+- Associated Press
+- Getty Images</t>
         </is>
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>1. Felipe Massa crashed in his last home Grand Prix because he couldn't handle the heavy rain.
-2. The race was suspended due to the heavy rain, making it difficult for drivers to maintain control of their vehicles.
-3. Massa's retirement was celebrated by his adoring fans, with many of them coming out to see his last race.
-4. The pits and rival teams showed their appreciation for Massa's contributions to the sport by giving him a guard of honor and a warm sendoff.
-5. The championship is still undecided as the race was won by Lewis Hamilton, but the overall winner will be determined in the next race.</t>
+          <t>The context does not provide any information about why the events described in the texts occurred, so I cannot answer this question from the provided context.</t>
         </is>
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>1. Felipe Massa, a popular and respected driver, announced his retirement from Formula One (F1) at the end of the season.
-2. His retirement was marked by his last home Grand Prix at Interlagos, where he raced for Williams.
-3. During the race, heavy rain caused poor visibility and made it difficult for drivers to maintain control of their cars.
-4. In lap 48, Massa's car crashed due to the poor weather conditions.
-5. The crowd, which was full of adoring fans, reacted with shock and dismay at the crash.
-6. Massa walked out of the car and the track, visibly emotional and overwhelmed by the support he received from his home crowd.
-7. Despite the crash, Massa was given a guard of honour by rival teams as he left the pit lane.
-8. The pits and pit crews paid tribute to Massa, showing their appreciation for his dedication and contribution to the sport.
-9. Lewis Hamilton won the race in dangerous conditions, with several other drivers also experiencing crashes or near-misses.
-10. The championship remains und</t>
+          <t>The events described in the texts are:
+1. Felipe Massa crashed his Williams car in lap 48 at the Grand Prix in Interlagos, Brazil.
+2. The crash caused damage to his car and he was unable to finish the race.
+3. Massa fought back tears as he was overwhelmed by the emotion coming from his home crowd.
+4. He said thank you very much to his fans, his team, and his country for supporting him throughout his career.
+5. He was given a guard of honour as he walked to meet his wife and son.
+6. Lewis Hamilton won a dangerous Grand Prix that saw a number of cars aquaplaning across the track.</t>
         </is>
       </c>
     </row>
@@ -1351,84 +1206,55 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>1. Teenage F1 star Max Verstappen spins his car at 180mph during dangerous conditions at the Brazilian Grand Prix.
-2. Verstappen clips the curb on the entrance to the home straight, causing his car to spin sideways and slide down the track.
-3. The back of Verstappen's car slides out, pointing towards the barrier, but he manages to straighten up and avoid a serious accident.
-4. Verstappen's incredible recovery earns him third place in the Grand Prix.
-5. Verstappen's aggressive driving style is praised and criticized.
-6. The young Dutchman gains universal praise for avoiding a serious accident during hazardous conditions.
-7. Max Verstappen's father was also a Formula One driver.
-8. Verstappen made his F1 debut at the age of 17 for Toro Rosso.
-9. Verstappen has won one race and has six podium finishes in his career.
-10. Verstappen currently ranks fifth in the drivers' championship standings.
-11. The safety car was deployed</t>
+          <t>Sure, here's a list of events that occur in the text:
+1. Max Verstappen loses control of his car as he clips the curb on the entrance to the long home straight, spinning his car sideways and sliding dangerously down the track.
+2. Verstappen produces an incredible display to finish third at the Brazilian Grand Prix.
+3. A number of spectacular crashes caused major delays as drivers struggled to cope with the wet weather.
+4. Verstappen is one of the hottest teenage talents F1 has ever seen and in his two seasons in the sport has thrilled and frustrated in equal measure, with an aggressive driving style which has split opinion both in the pits and in the stands.
+5. Verstappen avoids a serious accident in hazardous conditions in Brazil, during a race in which a number of spectacular crashes caused major delays as drivers struggled to cope with the wet weather.
+6. Verstappen is able to straighten up and regain control.
+7. He gains universal praise for the way he avoided a serious accident in hazardous conditions in Brazil, during a race in which a number of spectacular crashes caused major delays as drivers struggled to cope with the wet weather.</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Brazil: São Paulo: Interlagos</t>
+          <t>The events described in the text occurred at the Brazilian Grand Prix.
+- Interlagos Circuit
+1. Brazil</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>1. 2017-09-22 - Verstappen spins out at high speed at the Brazilian Grand Prix.
-2. 2017-09-24 - Verstappen manages to avoid a serious accident and finishes third in the Brazilian Grand Prix.
-3. 2017-11-26 - Hamilton wins the Brazilian Grand Prix, maintaining his chances of winning the world championship.
-4. 2017-11-27 - Abu Dhabi Grand Prix, the final race of the season.</t>
+          <t>The context does not specify a specific date, so I cannot answer this question from the provided context.</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>1. Max Verstappen
-2. Red Bull
-3. F1 (Formula One)
-4. Lewis Hamilton
-5. Nico Rosberg
-6. Toro Rosso
-7. Sebastian Vettel
-8. Kimi Raikkonen
-9. Felipe Massa
-10. Ayrton Senna
-11. Mercedes
-12. Ferrari
-13. Interlagos circuit
-14. Brazilian Grand Prix
-15. Ayrton Senna
-16. Abu Dhabi
-17. Yellow flags
-18. Red flags
-19. Toro Rosso
-20. Mercedes
-21. Ferrari
-22. F1 race organisers
-23. F1 drivers
-24. F1 fans
-25. F1 pits crew
-26. F1 team radio</t>
+          <t>Sure! Here is a list of people and organizations mentioned in the text:
+1. Max Verstappen
+2. Jos Verstappen
+3. Toro Rosso
+4. Formula One
+5. Sebastian Vettel
+6. Kimi Raikkonen
+7. Felipe Massa
+8. Lewis Hamilton
+9. Nico Rosberg</t>
         </is>
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>1. Max Verstappen spun his car at 180mph: The young driver lost control of his car as he clipped the curb on the entrance to the long home straight, causing his car to spin sideways and slide down the track.
-2. Verstappen avoided a serious accident: Despite spinning at high speed in dangerous conditions, Verstappen was able to regain control of his car and avoid hitting the wall of the track or any other cars.
-3. The Brazilian Grand Prix faced several crashes: The wet weather made it difficult for drivers to maintain control of their cars, leading to multiple crashes throughout the race, causing delays and interruptions.
-4. Safety cars were deployed: To manage the crashes and ensure driver safety, the race officials brought out safety cars several times to lead the drivers around the track at a slower pace.
-5. Red flags were produced: The race organizers had to stop the race twice due to hazardous conditions, such as heavy rain and standing water, that made it impossible for drivers to race safely.
-6. Drivers called for the race to be abandoned: Some drivers, including Sebastian Vettel, were frustrated with the</t>
+          <t>The events described in the text occurred because of the heavy rain that was falling during the race. The rain made the track slippery and dangerous, which caused many drivers to lose control of their cars and spin out.</t>
         </is>
       </c>
       <c r="M10" t="inlineStr">
         <is>
-          <t>1. Verstappen spun his car at 180mph in dangerous conditions.
-2. He clipped the curb on the entrance to the long home straight.
-3. His car slid dangerously down the track.
-4. He was able to straighten up and regain control.
-5. He finished third in the Brazilian Grand Prix.
-6. There were five safety car deployments and two red flag incidents during the race.
-7. Hamilton won the race from pole position and maintained his chances of winning the championship.
-8. Raikkonen and Massa crashed out of the race, causing delays and safety concerns.
-9. Verstappen's aggressive driving style split opinion among the pit crews and spectators.
-10. The race organisers faced criticism for the handling of safety measures during the hazardous conditions.</t>
+          <t>Sure, here is the list of events that occurred:
+1. Teenage Formula One star Max Verstappen showed nerves of steel as he somehow managed to avoid a serious accident despite spinning his car at 180mph in dangerous conditions at the Brazilian Grand Prix.
+2. Verstappen lost control as he clipped the curb on the entrance to the long home straight, spinning his car sideways and sliding dangerously down the track.
+3. Despite clipping the curb, Verstappen was able to straighten up and regain control.
+4. Verstappen produced an incredible display to finish third at the Brazilian Grand Prix.
+5. After the incident, Verstappen's team calmly said, "well held Max, well held", on the team radio before the driver himself joked, "my heartbeat went a little higher there."</t>
         </is>
       </c>
     </row>
@@ -1470,66 +1296,61 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>1. The British Transport Police and emergency services were called to the scene of a derailed tram near London.
-2. Seven people were confirmed dead as a result of the incident.
-3. At least 51 people were taken to the hospital for treatment of injuries sustained in the accident.
-4. The London Ambulance Service's hazardous area response team was sent to the site of the accident.
-5. The driver of the tram was arrested by the police.
-6. The cause of the accident was unknown, and an investigation was launched.
-7. People trapped inside the tram were freed by emergency services during the morning.</t>
+          <t>Sure, here is a list of events that occur in the text:
+1. A tram derailed near London on Wednesday.
+2. At least seven people were killed and dozens more were injured when the tram derailed near London.
+3. The driver of the tram has been arrested.
+4. The police were called to the scene in Croydon, south of the British capital, shortly after 6 a.m.
+5. Officers, firefighters and paramedics worked through the morning to free people who were trapped inside the tram.
+6. At least seven people are now confirmed as having died as a result of the incident.
+7. The cause of the accident was unclear, the police said.
+8. An investigation was opened.</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t xml:space="preserve"> England, United Kingdom, Croydon</t>
+          <t>The events occurred near London, England.
+1. Croydon, South of London.</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 1. The police were called to the scene in Croydon: 2016-11-09
-2. The accident took place: 2016-11-09
-3. The injured were treated at the scene: 2016-11-09
-4. The injured were taken to the hospital: 2016-11-09
-5. The London Ambulance Service sent its hazardous area response team to the site of the accident: 2016-11-09</t>
+          <t>The events described in the text occurred on Wednesday, [yyyy-mm-dd].
+1. A tram derailed near London on Wednesday, [yyyy-mm-dd].
+2. The driver of the tram has been arrested.
+3. At least seven people were killed and dozens more were injured.</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 1. People:
-a. The driver of the tram
-b. At least seven people who died
-c. Dozens more who were injured
-d. The passengers of the tram
-e. The emergency services personnel (police, firefighters, paramedics)
-f. The staff of the London Ambulance Service
-g. Unnamed people who were treated at the scene
-2. Organizations:
-a. British Transport Police
-b. London Ambulance Service
-c. British police
-d. Emergency services (police, firefighters, paramedics)
-e. London Ambulance Service's hazardous area response team
-f. The hospital where the injured were taken</t>
+          <t>Sure, here is the list of people and organizations described in the text:
+**People:**
+1. Driver of the tram
+2. Police officers
+3. Firefighters
+4. Paramedics
+5. Peter McKenna, the deputy director of operations for the London Ambulance Service
+**Organizations:**
+1. British police
+2. British Transport Police</t>
         </is>
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>1. A tram derailed near London, causing multiple casualties.
-2. At least seven people died and dozens more were injured in the incident.
-3. The driver of the tram was arrested by the police.
-4. The British Transport Police, London Ambulance Service, and other emergency services responded to the scene.
-5. An investigation into the cause of the accident was launched.</t>
+          <t>The context does not provide a reason for why the events described in the texts occurred, so I cannot answer this question from the provided context.</t>
         </is>
       </c>
       <c r="M11" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 1. The police were called to the scene in Croydon, south of London, after a tram derailed.
-2. Emergency services, including the police, firefighters, and paramedics, responded to the incident.
-3. The police confirmed that at least seven people died as a result of the tram accident.
-4. The London Ambulance Service sent a hazardous area response team to the site.
-5. A total of 51 injured people were taken to the hospital for treatment.
-6. The driver of the tram was arrested.
-7. An investigation into the cause of the accident was launched.</t>
+          <t>Sure, here's a summary of the events that occurred:
+1. A tram derailed near London on Wednesday.
+2. At least seven people were killed and dozens more were injured.
+3. The driver of the tram has been arrested.
+4. The police were called to the scene in Croydon, south of the British capital, shortly after 6 a.m.
+5. Officers, firefighters and paramedics worked through the morning to free people who were trapped inside the tram.
+6. At least seven people are now confirmed as having died as a result of the incident.
+7. The cause of the accident was unclear.
+8. An investigation was opened.</t>
         </is>
       </c>
     </row>

</xml_diff>